<commit_message>
Added colum in excel sheet
</commit_message>
<xml_diff>
--- a/input/requirements/PractitionerRole.xlsx
+++ b/input/requirements/PractitionerRole.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edelman_nict1\IGs\GBB-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33A396DF-650A-437F-A70B-931D3A5A436E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E933D0-4D74-45B5-8547-AAB19E8C6AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="655" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="655" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="3" r:id="rId1"/>
@@ -2263,154 +2263,155 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44D01FA7-4587-470D-A390-D8587FD365B7}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B1:E14"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.42578125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="107.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="70.42578125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="9.109375" style="2"/>
+    <col min="2" max="2" width="23.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.44140625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="107.33203125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="70.44140625" style="2" customWidth="1"/>
+    <col min="6" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="D1" s="12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+    <row r="2" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="9" t="s">
+      <c r="C2" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="3" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B3" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="C3" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="87" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="2:5" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="2:5" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="C5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="D5" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+    <row r="6" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B6" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="C6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="D6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="E6" s="19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+    <row r="7" spans="2:5" ht="62.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="C7" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="138.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+    <row r="8" spans="2:5" ht="138.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="9" t="s">
+      <c r="C8" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="3"/>
-    </row>
-    <row r="10" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B9" s="8"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B10" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="19" t="s">
+      <c r="D10" s="19" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+    <row r="11" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B11" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="19" t="s">
+      <c r="D11" s="19" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="75" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
+    <row r="12" spans="2:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="B12" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="18" t="s">
+      <c r="C12" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D12" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="8"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="8"/>
+    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B13" s="8"/>
+    </row>
+    <row r="14" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B14" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C11" r:id="rId1" xr:uid="{A15F1FB0-0D9C-4461-9E1E-58AFB253D7E2}"/>
-    <hyperlink ref="D6" r:id="rId2" xr:uid="{43CF51E7-BFF5-4D03-B360-14A771CE061E}"/>
+    <hyperlink ref="D11" r:id="rId1" xr:uid="{A15F1FB0-0D9C-4461-9E1E-58AFB253D7E2}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{43CF51E7-BFF5-4D03-B360-14A771CE061E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2419,20 +2420,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C04309E7-653D-4B76-B9C4-5CE689010C87}">
   <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="87.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="44.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="87.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="44.109375" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="48"/>
       <c r="B1" s="48"/>
       <c r="C1" s="29"/>
       <c r="D1" s="29"/>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="28"/>
       <c r="B2" s="30" t="s">
         <v>32</v>
@@ -2444,7 +2445,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="28"/>
       <c r="B3" s="31" t="s">
         <v>35</v>
@@ -2454,7 +2455,7 @@
       </c>
       <c r="D3" s="31"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="28"/>
       <c r="B4" s="29" t="s">
         <v>37</v>
@@ -2466,7 +2467,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="28"/>
       <c r="B5" s="31" t="s">
         <v>40</v>
@@ -2476,7 +2477,7 @@
       </c>
       <c r="D5" s="31"/>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="28"/>
       <c r="B6" s="29" t="s">
         <v>42</v>
@@ -2486,7 +2487,7 @@
       </c>
       <c r="D6" s="29"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="28"/>
       <c r="B7" s="31" t="s">
         <v>44</v>
@@ -2496,7 +2497,7 @@
       </c>
       <c r="D7" s="31"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="28"/>
       <c r="B8" s="29" t="s">
         <v>46</v>
@@ -2506,7 +2507,7 @@
       </c>
       <c r="D8" s="29"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="28"/>
       <c r="B9" s="31" t="s">
         <v>47</v>
@@ -2516,7 +2517,7 @@
       </c>
       <c r="D9" s="31"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="28"/>
       <c r="B10" s="29" t="s">
         <v>49</v>
@@ -2526,7 +2527,7 @@
       </c>
       <c r="D10" s="29"/>
     </row>
-    <row r="11" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="28"/>
       <c r="B11" s="31" t="s">
         <v>51</v>
@@ -2538,7 +2539,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="28"/>
       <c r="B12" s="29" t="s">
         <v>54</v>
@@ -2574,19 +2575,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1A0E3D-BE28-4965-A5FF-C835B3665CFB}">
   <dimension ref="B2:L10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="31" customWidth="1"/>
-    <col min="5" max="6" width="65.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="82.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="37.7109375" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="10" width="35.28515625" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="65.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="82.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="37.6640625" customWidth="1"/>
+    <col min="9" max="9" width="15.6640625" customWidth="1"/>
+    <col min="10" max="10" width="35.33203125" customWidth="1"/>
+    <col min="11" max="11" width="8.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B2" s="17" t="s">
         <v>56</v>
       </c>
@@ -2617,7 +2618,7 @@
       <c r="K2" s="5"/>
       <c r="L2" s="5"/>
     </row>
-    <row r="3" spans="2:12" s="23" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:12" s="23" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B3" s="14" t="s">
         <v>65</v>
       </c>
@@ -2643,7 +2644,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="4" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:12" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B4" s="14" t="s">
         <v>73</v>
       </c>
@@ -2666,7 +2667,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="2:12" s="23" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:12" s="23" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B5" s="14" t="s">
         <v>77</v>
       </c>
@@ -2690,7 +2691,7 @@
       </c>
       <c r="I5" s="10"/>
     </row>
-    <row r="6" spans="2:12" s="23" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:12" s="23" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B6" s="14" t="s">
         <v>82</v>
       </c>
@@ -2712,7 +2713,7 @@
       </c>
       <c r="I6" s="10"/>
     </row>
-    <row r="7" spans="2:12" s="26" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:12" s="26" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B7" s="14" t="s">
         <v>87</v>
       </c>
@@ -2736,7 +2737,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="8" spans="2:12" s="26" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:12" s="26" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="14" t="s">
         <v>92</v>
       </c>
@@ -2760,7 +2761,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="9" spans="2:12" s="26" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:12" s="26" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B9" s="14" t="s">
         <v>98</v>
       </c>
@@ -2784,7 +2785,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="14" t="s">
         <v>103</v>
       </c>
@@ -2813,26 +2814,26 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1E71E66-FD43-4603-91A3-4CCDD6133986}">
   <dimension ref="B2:H24"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.85546875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" style="4" customWidth="1"/>
+    <col min="1" max="1" width="3.88671875" style="4" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" style="4" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" style="4" customWidth="1"/>
     <col min="4" max="4" width="74" style="4" customWidth="1"/>
-    <col min="5" max="5" width="65.28515625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="24.42578125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="73.7109375" style="4" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="4"/>
+    <col min="5" max="5" width="65.33203125" style="4" customWidth="1"/>
+    <col min="6" max="6" width="24.44140625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="21.6640625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="73.6640625" style="4" customWidth="1"/>
+    <col min="9" max="16384" width="9.109375" style="4"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="27" t="s">
         <v>104</v>
       </c>
       <c r="F2" s="27"/>
     </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B3" s="15" t="s">
         <v>105</v>
       </c>
@@ -2849,7 +2850,7 @@
       <c r="G3" s="10"/>
       <c r="H3" s="10"/>
     </row>
-    <row r="4" spans="2:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B4" s="4" t="s">
         <v>108</v>
       </c>
@@ -2860,7 +2861,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="5" spans="2:8" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" ht="78" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>111</v>
       </c>
@@ -2874,7 +2875,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B6" s="4" t="s">
         <v>114</v>
       </c>
@@ -2885,7 +2886,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" ht="72" x14ac:dyDescent="0.3">
       <c r="B7" s="4" t="s">
         <v>116</v>
       </c>
@@ -2899,7 +2900,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>88</v>
       </c>
@@ -2913,7 +2914,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B9" s="4" t="s">
         <v>66</v>
       </c>
@@ -2927,12 +2928,12 @@
         <v>121</v>
       </c>
     </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B11" s="39" t="s">
         <v>123</v>
       </c>
@@ -2946,7 +2947,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B12" s="42" t="s">
         <v>126</v>
       </c>
@@ -2960,7 +2961,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B13" s="39" t="s">
         <v>108</v>
       </c>
@@ -2974,7 +2975,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B14" s="42" t="s">
         <v>127</v>
       </c>
@@ -2988,22 +2989,22 @@
         <v>125</v>
       </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B18" s="20"/>
       <c r="C18" s="20"/>
     </row>
-    <row r="19" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
       <c r="D19" s="13"/>
     </row>
-    <row r="20" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
     </row>
-    <row r="21" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B24" s="20"/>
       <c r="C24" s="20"/>
       <c r="D24" s="20"/>
@@ -3019,15 +3020,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D7E96EB-0EDF-43CA-9149-BA391692EDD0}">
   <dimension ref="B2:E12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="22.7109375" customWidth="1"/>
-    <col min="3" max="3" width="27.42578125" customWidth="1"/>
-    <col min="4" max="4" width="24.85546875" customWidth="1"/>
-    <col min="5" max="5" width="53.140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
+    <col min="3" max="3" width="27.44140625" customWidth="1"/>
+    <col min="4" max="4" width="24.88671875" customWidth="1"/>
+    <col min="5" max="5" width="53.109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
         <v>128</v>
       </c>
@@ -3041,7 +3042,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>132</v>
       </c>
@@ -3052,7 +3053,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>135</v>
       </c>
@@ -3060,7 +3061,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>137</v>
       </c>
@@ -3074,7 +3075,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>141</v>
       </c>
@@ -3088,7 +3089,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>144</v>
       </c>
@@ -3099,7 +3100,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>146</v>
       </c>
@@ -3110,7 +3111,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>149</v>
       </c>
@@ -3121,7 +3122,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>150</v>
       </c>
@@ -3129,7 +3130,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B12" s="44" t="s">
         <v>152</v>
       </c>
@@ -3145,17 +3146,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{688495E5-0C43-4F64-B944-96A9F5BA516C}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" style="1" customWidth="1"/>
     <col min="2" max="2" width="39" style="1" customWidth="1"/>
     <col min="3" max="3" width="33" style="1" customWidth="1"/>
-    <col min="4" max="4" width="81.140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" style="1" customWidth="1"/>
-    <col min="6" max="7" width="54.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="81.109375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.44140625" style="1" customWidth="1"/>
+    <col min="6" max="7" width="54.6640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="168.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="168.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="36" t="s">
         <v>153</v>
       </c>
@@ -3178,7 +3179,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="195" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="37" t="s">
         <v>156</v>
       </c>
@@ -3201,7 +3202,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>163</v>
       </c>
@@ -3224,7 +3225,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>169</v>
       </c>
@@ -3241,7 +3242,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>163</v>
       </c>
@@ -3261,7 +3262,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>163</v>
       </c>
@@ -3284,7 +3285,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>163</v>
       </c>
@@ -3304,7 +3305,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="8" spans="1:8" s="23" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" s="23" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="10" t="s">
         <v>163</v>
       </c>
@@ -3326,7 +3327,7 @@
       </c>
       <c r="H8" s="10"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="45" t="s">
         <v>163</v>
       </c>
@@ -3346,7 +3347,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="C11"/>
     </row>
   </sheetData>
@@ -3365,7 +3366,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8748DCD5-A959-41F5-9A2D-B277CB3E46A1}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3373,26 +3374,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -3599,10 +3580,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3619,20 +3631,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Added row above the table
</commit_message>
<xml_diff>
--- a/input/requirements/PractitionerRole.xlsx
+++ b/input/requirements/PractitionerRole.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2E933D0-4D74-45B5-8547-AAB19E8C6AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2ECE55D6-70C8-43E7-AD92-EFB723A1F541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="655" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
@@ -2263,7 +2263,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44D01FA7-4587-470D-A390-D8587FD365B7}">
-  <dimension ref="B1:E14"/>
+  <dimension ref="B2:E15"/>
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.109375" style="2"/>
@@ -2274,144 +2274,144 @@
     <col min="6" max="16384" width="9.109375" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B1" s="6" t="s">
+    <row r="2" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C2" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B2" s="7" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B3" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="2:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="B4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C4" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="2:5" ht="87" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="7" t="s">
+    <row r="5" spans="2:5" ht="87" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="2:5" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="7" t="s">
+    <row r="6" spans="2:5" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C6" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D6" s="11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B6" s="7" t="s">
+    <row r="7" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B7" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C7" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D7" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E7" s="19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="2:5" ht="62.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="7" t="s">
+    <row r="8" spans="2:5" ht="62.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="2:5" ht="138.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="7" t="s">
+    <row r="9" spans="2:5" ht="138.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" s="8"/>
-      <c r="C9" s="3"/>
-    </row>
-    <row r="10" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B10" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="19" t="s">
-        <v>189</v>
-      </c>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B10" s="8"/>
+      <c r="C10" s="3"/>
     </row>
     <row r="11" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="7" t="s">
+        <v>188</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D11" s="19" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="12" spans="2:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D12" s="19" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="2:5" ht="72" x14ac:dyDescent="0.3">
-      <c r="B12" s="7" t="s">
+    <row r="13" spans="2:5" ht="72" x14ac:dyDescent="0.3">
+      <c r="B13" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C13" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B13" s="8"/>
     </row>
     <row r="14" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B14" s="8"/>
     </row>
+    <row r="15" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="B15" s="8"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D11" r:id="rId1" xr:uid="{A15F1FB0-0D9C-4461-9E1E-58AFB253D7E2}"/>
-    <hyperlink ref="E6" r:id="rId2" xr:uid="{43CF51E7-BFF5-4D03-B360-14A771CE061E}"/>
+    <hyperlink ref="D12" r:id="rId1" xr:uid="{A15F1FB0-0D9C-4461-9E1E-58AFB253D7E2}"/>
+    <hyperlink ref="E7" r:id="rId2" xr:uid="{43CF51E7-BFF5-4D03-B360-14A771CE061E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3374,6 +3374,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -3580,27 +3600,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3617,23 +3636,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C46046CF-AC59-4D6A-A325-5977C53DC9DA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
PractitionerRole: changed IB tab for variability and availablitiy
</commit_message>
<xml_diff>
--- a/input/requirements/PractitionerRole.xlsx
+++ b/input/requirements/PractitionerRole.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\GBB-IG\input\requirements\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Nictiz\GBB-IG\input\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75AF215-0356-45B6-8AA2-616945301357}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07941A22-D065-4FBE-9EED-9FF4389603DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" tabRatio="655" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="655" activeTab="2" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="18" r:id="rId1"/>
@@ -50,17 +50,17 @@
   <commentList>
     <comment ref="D2" authorId="0" shapeId="0" xr:uid="{812FD7AE-C33E-4098-9678-0004F1C27ED0}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     Vanuit Xt-EHR alleen naamgegevens 0..1, de rest 0..*</t>
       </text>
     </comment>
     <comment ref="G2" authorId="1" shapeId="0" xr:uid="{5343DF36-C9C0-470B-A9B1-08DF05F31D2D}">
       <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
+        <t>[Opmerkingenthread]
+U kunt deze opmerkingenthread lezen in uw versie van Excel. Eventuele wijzigingen aan de thread gaan echter verloren als het bestand wordt geopend in een nieuwere versie van Excel. Meer informatie: https://go.microsoft.com/fwlink/?linkid=870924
+Opmerking:
     eOverdracht als basis gebruikt, aanvullend ook zibs2020, zibs2026 en Xt-EHR/EU-Core geraadpleegd</t>
       </text>
     </comment>
@@ -69,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="176">
   <si>
     <t>Veld</t>
   </si>
@@ -268,9 +268,6 @@
 Het betreft hierbij de erkende medische specialismen zoals vermeld in de wet BIG. Bijvoorbeeld huisarts of cardioloog. </t>
   </si>
   <si>
-    <t>AGB en UZI zijn geprefereerde codesystemen voor nederlandse zorgverleners</t>
-  </si>
-  <si>
     <t>0..*</t>
   </si>
   <si>
@@ -306,9 +303,6 @@
   </si>
   <si>
     <t>0..1</t>
-  </si>
-  <si>
-    <t>ZVL-012</t>
   </si>
   <si>
     <t>availableTime - PractitionerRole.availabletime</t>
@@ -638,6 +632,21 @@
   </si>
   <si>
     <t>https://hl7.org/fhir/R4/practitionerrole.html</t>
+  </si>
+  <si>
+    <t>(coded)</t>
+  </si>
+  <si>
+    <t>(reference GBB-ContactPoint)</t>
+  </si>
+  <si>
+    <t>(reference GBB-Organization)</t>
+  </si>
+  <si>
+    <t>(reference GBB-Practitioner)</t>
+  </si>
+  <si>
+    <t>(coded) AGB en UZI zijn geprefereerde codesystemen voor nederlandse zorgverleners</t>
   </si>
 </sst>
 </file>
@@ -883,7 +892,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -995,141 +1004,40 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="2" xr:uid="{B0F7F417-6139-AC4A-9919-70BAFABB9069}"/>
   </cellStyles>
   <dxfs count="29">
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFCC"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFFCC"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="5"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-      <border diagonalUp="0" diagonalDown="0" outline="0">
-        <left style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </left>
-        <right style="thin">
-          <color theme="5" tint="-0.249977111117893"/>
-        </right>
-        <top/>
-        <bottom/>
-      </border>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment wrapText="1"/>
-    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -1296,6 +1204,126 @@
         </patternFill>
       </fill>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFFFCC"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0" outline="0">
+        <left style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </left>
+        <right style="thin">
+          <color theme="5" tint="-0.249977111117893"/>
+        </right>
+        <top/>
+        <bottom/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1906,46 +1934,46 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="A2:H10" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
-  <autoFilter ref="A2:H10" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="A2:H9" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="A2:H9" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Aanwezigheid" dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Verleden/heden/toekomst" dataDxfId="18" dataCellStyle="Hyperlink"/>
-    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Herkomst" dataDxfId="17" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Opmerkingen" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Aanwezigheid" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Verleden/heden/toekomst" dataDxfId="2" dataCellStyle="Hyperlink"/>
+    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Herkomst" dataDxfId="1" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Opmerkingen" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7CF12276-5DB5-4F90-8695-E8C211C8F244}" name="Tabel5" displayName="Tabel5" ref="A1:G9" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7CF12276-5DB5-4F90-8695-E8C211C8F244}" name="Tabel5" displayName="Tabel5" ref="A1:G9" totalsRowShown="0" headerRowDxfId="25" dataDxfId="24">
   <autoFilter ref="A1:G9" xr:uid="{7CF12276-5DB5-4F90-8695-E8C211C8F244}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B97F8D91-3082-4CC3-88C3-3AFD25565086}" name="Actie" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{D7C302FA-9136-48F1-8EB1-623FD7B82D0B}" name="Notitie" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{23C47ECA-78A1-46D2-B459-2ED9F0CD69F7}" name="Naam" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{0A87635E-2235-40AA-829B-E1ECCB1E6C33}" name="Omschrijving" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{263135AB-3C6A-4909-9685-2C2C6DED9D81}" name="Variabiliteit" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{698F8C8C-D318-4E44-AD77-5EB91FEF4EFA}" name="Aanwezigheid" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{06FAC50A-4314-452E-8D2E-120AF7C1D687}" name="Herkomst" dataDxfId="7"/>
+    <tableColumn id="1" xr3:uid="{B97F8D91-3082-4CC3-88C3-3AFD25565086}" name="Actie" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{D7C302FA-9136-48F1-8EB1-623FD7B82D0B}" name="Notitie" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{23C47ECA-78A1-46D2-B459-2ED9F0CD69F7}" name="Naam" dataDxfId="21"/>
+    <tableColumn id="4" xr3:uid="{0A87635E-2235-40AA-829B-E1ECCB1E6C33}" name="Omschrijving" dataDxfId="20"/>
+    <tableColumn id="5" xr3:uid="{263135AB-3C6A-4909-9685-2C2C6DED9D81}" name="Variabiliteit" dataDxfId="19"/>
+    <tableColumn id="6" xr3:uid="{698F8C8C-D318-4E44-AD77-5EB91FEF4EFA}" name="Aanwezigheid" dataDxfId="18"/>
+    <tableColumn id="7" xr3:uid="{06FAC50A-4314-452E-8D2E-120AF7C1D687}" name="Herkomst" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}" name="Tabel362" displayName="Tabel362" ref="B3:E18" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}" name="Tabel362" displayName="Tabel362" ref="B3:E18" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="B3:E18" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2FB2A545-3E03-42E2-A7C5-CBA6BF51E763}" name="Data element" dataDxfId="4"/>
-    <tableColumn id="2" xr3:uid="{B3874943-8B88-43AA-B0A0-4B5081B45198}" name="Informatiestandaard" dataDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{4FFBC5A0-455F-4C81-8A81-963E0DD492F2}" name="Uitleg" dataDxfId="2"/>
-    <tableColumn id="4" xr3:uid="{98900A9D-2F8F-43EC-A740-2203C6F18585}" name="Uitkomst" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{2FB2A545-3E03-42E2-A7C5-CBA6BF51E763}" name="Data element" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{B3874943-8B88-43AA-B0A0-4B5081B45198}" name="Informatiestandaard" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{4FFBC5A0-455F-4C81-8A81-963E0DD492F2}" name="Uitleg" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{98900A9D-2F8F-43EC-A740-2203C6F18585}" name="Uitkomst" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1958,7 +1986,7 @@
     <tableColumn id="1" xr3:uid="{E1FF28EC-54D9-4C5E-B216-CE683489BB36}" name="EN name"/>
     <tableColumn id="2" xr3:uid="{9E77889B-1E8C-4DC1-8285-9B73CD19BE32}" name="NL name"/>
     <tableColumn id="3" xr3:uid="{3EC0721C-3350-474C-924F-1C725876433A}" name="FHIR destination"/>
-    <tableColumn id="4" xr3:uid="{47E45A34-8D1A-4889-AE01-49B829C6B42C}" name="Toelichting" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{47E45A34-8D1A-4889-AE01-49B829C6B42C}" name="Toelichting" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2293,24 +2321,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF696AA-9F2F-43BC-962B-71A16984DFB4}">
   <dimension ref="A1:E23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="52.109375" customWidth="1"/>
+    <col min="2" max="2" width="52.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="190.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="190.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1"/>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="43" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="42" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2318,7 +2346,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2327,7 +2355,7 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="90" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -2336,7 +2364,7 @@
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>8</v>
       </c>
@@ -2345,7 +2373,7 @@
       </c>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -2354,7 +2382,7 @@
       </c>
       <c r="E7" s="2"/>
     </row>
-    <row r="8" spans="1:5" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -2363,7 +2391,7 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" ht="201.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" ht="225" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>14</v>
       </c>
@@ -2372,47 +2400,47 @@
       </c>
       <c r="C9" s="2"/>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>163</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="C10" s="2"/>
+    </row>
+    <row r="11" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>165</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B11" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="C10" s="2"/>
-    </row>
-    <row r="11" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>167</v>
-      </c>
-      <c r="B11" s="12" t="s">
-        <v>168</v>
-      </c>
       <c r="C11" s="2"/>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B12" s="12"/>
       <c r="C12" s="2"/>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>167</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>168</v>
+      </c>
+      <c r="C13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>169</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B14" s="12" t="s">
         <v>170</v>
       </c>
-      <c r="C13" s="2"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>171</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>172</v>
-      </c>
       <c r="C14" s="2"/>
     </row>
-    <row r="15" spans="1:5" ht="129.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" ht="135" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -2421,35 +2449,35 @@
       </c>
       <c r="C15" s="22"/>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B16" s="12"/>
       <c r="C16" s="22"/>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B17" s="44"/>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" s="43"/>
       <c r="C17" s="22"/>
     </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="12"/>
       <c r="C18" s="22"/>
     </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" s="12"/>
       <c r="C19" s="22"/>
     </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B20" s="44"/>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B20" s="43"/>
       <c r="C20" s="22"/>
     </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B21" s="44"/>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B21" s="43"/>
       <c r="C21" s="22"/>
     </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B22" s="44"/>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B22" s="43"/>
       <c r="C22" s="22"/>
     </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" s="12"/>
       <c r="C23" s="22"/>
     </row>
@@ -2465,19 +2493,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C04309E7-653D-4B76-B9C4-5CE689010C87}">
   <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="26.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="87.5546875" style="1" customWidth="1"/>
-    <col min="3" max="3" width="44.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="87.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="44.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="21"/>
       <c r="B1" s="22"/>
       <c r="C1" s="22"/>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="23" t="s">
         <v>18</v>
       </c>
@@ -2488,7 +2516,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
         <v>21</v>
       </c>
@@ -2497,7 +2525,7 @@
       </c>
       <c r="C3" s="24"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="22" t="s">
         <v>23</v>
       </c>
@@ -2508,7 +2536,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
         <v>26</v>
       </c>
@@ -2517,7 +2545,7 @@
       </c>
       <c r="C5" s="24"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="22" t="s">
         <v>28</v>
       </c>
@@ -2526,7 +2554,7 @@
       </c>
       <c r="C6" s="22"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="24" t="s">
         <v>30</v>
       </c>
@@ -2535,7 +2563,7 @@
       </c>
       <c r="C7" s="24"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="22" t="s">
         <v>32</v>
       </c>
@@ -2544,7 +2572,7 @@
       </c>
       <c r="C8" s="22"/>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="24" t="s">
         <v>33</v>
       </c>
@@ -2553,7 +2581,7 @@
       </c>
       <c r="C9" s="24"/>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="22" t="s">
         <v>35</v>
       </c>
@@ -2562,7 +2590,7 @@
       </c>
       <c r="C10" s="22"/>
     </row>
-    <row r="11" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="24" t="s">
         <v>37</v>
       </c>
@@ -2573,7 +2601,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="22" t="s">
         <v>40</v>
       </c>
@@ -2604,21 +2632,21 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1A0E3D-BE28-4965-A5FF-C835B3665CFB}">
-  <dimension ref="A2:J10"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:J9"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31" customWidth="1"/>
-    <col min="3" max="3" width="65.6640625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="16.44140625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="44.88671875" style="1" customWidth="1"/>
-    <col min="6" max="6" width="37.6640625" customWidth="1"/>
-    <col min="7" max="7" width="15.6640625" customWidth="1"/>
-    <col min="8" max="8" width="35.33203125" customWidth="1"/>
-    <col min="9" max="9" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.7109375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="55.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="44.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="37.7109375" customWidth="1"/>
+    <col min="7" max="7" width="58.140625" customWidth="1"/>
+    <col min="8" max="8" width="35.28515625" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
         <v>42</v>
       </c>
@@ -2646,7 +2674,7 @@
       <c r="I2" s="4"/>
       <c r="J2" s="4"/>
     </row>
-    <row r="3" spans="1:10" s="16" customFormat="1" ht="72" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" s="16" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>50</v>
       </c>
@@ -2656,150 +2684,137 @@
       <c r="C3" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D3" s="41" t="s">
+      <c r="D3" s="51" t="s">
+        <v>175</v>
+      </c>
+      <c r="E3" s="49" t="s">
         <v>53</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="41"/>
+      <c r="G3" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="F3" s="42"/>
-      <c r="G3" s="15" t="s">
+    </row>
+    <row r="4" spans="1:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
         <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
-        <v>56</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>51</v>
       </c>
       <c r="C4" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="41"/>
+      <c r="G4" s="15" t="s">
         <v>57</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="5" t="s">
+    </row>
+    <row r="5" spans="1:10" s="16" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="50" t="s">
+        <v>172</v>
+      </c>
+      <c r="E5" s="49" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="41"/>
+      <c r="G5" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="F4" s="42"/>
-      <c r="G4" s="15" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" s="16" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="C5" s="5" t="s">
+    </row>
+    <row r="6" spans="1:10" s="16" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="D5" s="7"/>
-      <c r="E5" s="5" t="s">
+      <c r="B6" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="F6" s="41"/>
+      <c r="G6" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="F5" s="42"/>
-      <c r="G5" s="15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="16" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C6" s="5" t="s">
+    </row>
+    <row r="7" spans="1:10" s="19" customFormat="1" ht="68.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="50" t="s">
+        <v>171</v>
+      </c>
+      <c r="E7" s="50" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="41"/>
+      <c r="G7" s="10" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="19" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="E8" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="7"/>
-      <c r="E6" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="F6" s="42"/>
-      <c r="G6" s="15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" s="19" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="7"/>
-      <c r="E7" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="F7" s="42"/>
-      <c r="G7" s="10" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" s="19" customFormat="1" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" s="42"/>
+      <c r="F8" s="41"/>
       <c r="G8" s="10" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" s="19" customFormat="1" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="A9" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="C9" t="s">
-        <v>76</v>
-      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
       <c r="D9" s="7"/>
-      <c r="E9" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="F9" s="42"/>
-      <c r="G9" s="10" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="42"/>
-      <c r="G10" s="10"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="41"/>
+      <c r="G9" s="10"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="G7" r:id="rId1" xr:uid="{FEB7522F-2A9D-49C2-82F5-222BEE2F9415}"/>
-    <hyperlink ref="G8" r:id="rId2" xr:uid="{708A4C80-C2CD-48E7-8282-4E696A81C206}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId3"/>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId4"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
@@ -2807,22 +2822,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{688495E5-0C43-4F64-B944-96A9F5BA516C}">
   <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19" style="1" customWidth="1"/>
     <col min="2" max="2" width="39" style="1" customWidth="1"/>
     <col min="3" max="3" width="33" style="1" customWidth="1"/>
-    <col min="4" max="4" width="81.109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="14.44140625" style="1" customWidth="1"/>
-    <col min="6" max="7" width="54.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="81.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="54.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="168.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="168.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="29" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B1" s="29" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C1" s="29" t="s">
         <v>43</v>
@@ -2840,175 +2855,175 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="187.2" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" ht="195" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="30" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="D2" s="30" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="E2" s="30" t="s">
         <v>82</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="F2" s="30" t="s">
         <v>83</v>
       </c>
-      <c r="E2" s="30" t="s">
+      <c r="G2" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="F2" s="30" t="s">
+    </row>
+    <row r="3" spans="1:8" ht="135" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="G2" s="30" t="s">
+      <c r="B3" s="1" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="E3" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="G3" s="40" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="40" t="s">
+      <c r="B4" s="1" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="E4" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="G4" s="40" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" s="40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="1" t="s">
+      <c r="D5" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="E5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G5" s="40" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="C6" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G5" s="40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B6" s="1" t="s">
+      <c r="D6" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="E6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="G6" s="40" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="F6" s="1" t="s">
+      <c r="C7" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="G6" s="40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="E7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="40" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="16" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="C8" s="5" t="s">
         <v>105</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="G7" s="40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="16" customFormat="1" ht="66.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="C8" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>108</v>
-      </c>
       <c r="E8" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F8" s="14"/>
       <c r="G8" s="40" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="H8" s="5"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="38" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B9" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="38" t="s">
+        <v>108</v>
+      </c>
+      <c r="D9" s="39" t="s">
         <v>109</v>
       </c>
-      <c r="C9" s="38" t="s">
-        <v>110</v>
-      </c>
-      <c r="D9" s="39" t="s">
-        <v>111</v>
-      </c>
       <c r="E9" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G9" s="40" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C11"/>
     </row>
   </sheetData>
@@ -3026,208 +3041,234 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8748DCD5-A959-41F5-9A2D-B277CB3E46A1}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <dimension ref="A9:G9"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="47.7109375" customWidth="1"/>
+    <col min="2" max="2" width="80.28515625" customWidth="1"/>
+    <col min="6" max="6" width="71.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="9" spans="1:7" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="44" t="s">
+        <v>65</v>
+      </c>
+      <c r="B9" s="44" t="s">
+        <v>66</v>
+      </c>
+      <c r="C9" s="44"/>
+      <c r="D9" s="45" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" s="46"/>
+      <c r="F9" s="47" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="48"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="F9" r:id="rId1" xr:uid="{FEB7522F-2A9D-49C2-82F5-222BEE2F9415}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1E71E66-FD43-4603-91A3-4CCDD6133986}">
   <dimension ref="B2:H24"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.88671875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="22.44140625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="3.85546875" style="3" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" style="3" customWidth="1"/>
     <col min="4" max="4" width="74" style="3" customWidth="1"/>
-    <col min="5" max="5" width="65.33203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="24.44140625" style="3" customWidth="1"/>
-    <col min="7" max="7" width="21.6640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="73.6640625" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="9.109375" style="3"/>
+    <col min="5" max="5" width="65.28515625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="24.42578125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" style="3" customWidth="1"/>
+    <col min="8" max="8" width="73.7109375" style="3" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" s="20"/>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B3" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="F2" s="20"/>
-    </row>
-    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B3" s="9" t="s">
+      <c r="D3" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="E3" s="17" t="s">
         <v>114</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>115</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>116</v>
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5"/>
       <c r="H3" s="5"/>
     </row>
-    <row r="4" spans="2:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:8" ht="60" x14ac:dyDescent="0.25">
       <c r="B4" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D4" s="5" t="s">
+    </row>
+    <row r="5" spans="2:8" ht="78" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="5" spans="2:8" ht="78" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="3" t="s">
+      <c r="D5" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="D5" s="5" t="s">
+    </row>
+    <row r="6" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="C6" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="2:8" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B6" s="3" t="s">
+    <row r="7" spans="2:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D6" s="3" t="s">
+      <c r="C7" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D7" s="7" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="7" spans="2:8" ht="72" x14ac:dyDescent="0.3">
-      <c r="B7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D7" s="7" t="s">
+    </row>
+    <row r="8" spans="2:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="B8" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="C8" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B8" s="3" t="s">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="E8" s="3" t="s">
+      <c r="C9" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" s="7" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="9" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D9" s="7" t="s">
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E9" s="3" t="s">
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B11" s="32" t="s">
         <v>133</v>
-      </c>
-    </row>
-    <row r="10" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B10" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="11" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B11" s="32" t="s">
-        <v>135</v>
       </c>
       <c r="C11" s="33" t="s">
         <v>35</v>
       </c>
       <c r="D11" s="33" t="s">
+        <v>134</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B12" s="35" t="s">
         <v>136</v>
-      </c>
-      <c r="E11" s="34" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B12" s="35" t="s">
-        <v>138</v>
       </c>
       <c r="C12" s="33" t="s">
         <v>35</v>
       </c>
       <c r="D12" s="36" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E12" s="31" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B13" s="32" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C13" s="33" t="s">
         <v>35</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E13" s="34" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="35" t="s">
         <v>137</v>
-      </c>
-    </row>
-    <row r="14" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B14" s="35" t="s">
-        <v>139</v>
       </c>
       <c r="C14" s="33" t="s">
         <v>35</v>
       </c>
       <c r="D14" s="36" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E14" s="31" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
     </row>
-    <row r="19" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
     </row>
-    <row r="20" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
     </row>
-    <row r="21" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
       <c r="D24" s="13"/>
@@ -3243,119 +3284,119 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D7E96EB-0EDF-43CA-9149-BA391692EDD0}">
   <dimension ref="B2:E12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="22.6640625" customWidth="1"/>
-    <col min="3" max="3" width="27.44140625" customWidth="1"/>
-    <col min="4" max="4" width="24.88671875" customWidth="1"/>
-    <col min="5" max="5" width="53.109375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="27.42578125" customWidth="1"/>
+    <col min="4" max="4" width="24.85546875" customWidth="1"/>
+    <col min="5" max="5" width="53.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" t="s">
+        <v>139</v>
+      </c>
+      <c r="D2" t="s">
         <v>140</v>
       </c>
-      <c r="C2" t="s">
+      <c r="E2" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="D2" t="s">
+    </row>
+    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
         <v>142</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="C3" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B3" t="s">
+      <c r="D3" t="s">
         <v>144</v>
       </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
         <v>145</v>
       </c>
-      <c r="D3" t="s">
+      <c r="C4" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" t="s">
+    <row r="5" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
         <v>147</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C5" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="5" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B5" t="s">
+      <c r="D5" t="s">
         <v>149</v>
       </c>
-      <c r="C5" t="s">
+      <c r="E5" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="D5" t="s">
+    </row>
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
         <v>151</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="C6" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B6" t="s">
+      <c r="D6" t="s">
         <v>153</v>
       </c>
-      <c r="C6" t="s">
+      <c r="E6" s="1" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
         <v>154</v>
       </c>
-      <c r="D6" t="s">
+      <c r="C7" t="s">
         <v>155</v>
       </c>
-      <c r="E6" s="1" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+      <c r="D7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="45" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>156</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C8" t="s">
         <v>157</v>
       </c>
-      <c r="D7" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="B8" t="s">
+      <c r="E8" s="1" t="s">
         <v>158</v>
       </c>
-      <c r="C8" t="s">
+    </row>
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
         <v>159</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="C9" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B9" t="s">
+      <c r="C10" t="s">
         <v>161</v>
       </c>
-      <c r="C9" t="s">
-        <v>161</v>
-      </c>
-      <c r="D9" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B10" t="s">
+    </row>
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B12" s="37" t="s">
         <v>162</v>
-      </c>
-      <c r="C10" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B12" s="37" t="s">
-        <v>164</v>
       </c>
     </row>
   </sheetData>
@@ -3367,26 +3408,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -3593,10 +3614,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
+    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3619,20 +3671,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
-    <ds:schemaRef ds:uri="06294a2e-6f87-4144-83b8-94a4d04d144a"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
PractitionerRole: refreshed requirements file
</commit_message>
<xml_diff>
--- a/input/requirements/PractitionerRole.xlsx
+++ b/input/requirements/PractitionerRole.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/PractitionerRole/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2824" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7EA8AE7-CAE3-432C-BE58-10C8FCFC50B8}"/>
+  <xr:revisionPtr revIDLastSave="3045" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4D37651-9E16-4768-8594-450EB93BF6B1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="655" firstSheet="2" activeTab="2" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" tabRatio="655" firstSheet="2" activeTab="6" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
-    <sheet name="Context" sheetId="3" r:id="rId1"/>
+    <sheet name="Concept" sheetId="18" r:id="rId1"/>
     <sheet name="Bronnen" sheetId="17" r:id="rId2"/>
     <sheet name="Informatiebehoefte" sheetId="12" r:id="rId3"/>
-    <sheet name="Ter discussie" sheetId="2" r:id="rId4"/>
-    <sheet name="Mapping rolcodelijst" sheetId="14" r:id="rId5"/>
-    <sheet name="Ongedekte informatiebehoefte" sheetId="15" r:id="rId6"/>
-    <sheet name="Overwegingen voor de toekomst" sheetId="16" r:id="rId7"/>
+    <sheet name="Ongedekte informatiebehoefte" sheetId="15" r:id="rId4"/>
+    <sheet name="Overwegingen voor de toekomst" sheetId="16" r:id="rId5"/>
+    <sheet name="Ter discussie" sheetId="2" r:id="rId6"/>
+    <sheet name="Mapping rolcodelijst" sheetId="14" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,19 +44,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={812FD7AE-C33E-4098-9678-0004F1C27ED0}</author>
     <author>tc={5343DF36-C9C0-470B-A9B1-08DF05F31D2D}</author>
   </authors>
   <commentList>
-    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{812FD7AE-C33E-4098-9678-0004F1C27ED0}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Vanuit Xt-EHR alleen naamgegevens 0..1, de rest 0..*</t>
-      </text>
-    </comment>
-    <comment ref="I2" authorId="1" shapeId="0" xr:uid="{5343DF36-C9C0-470B-A9B1-08DF05F31D2D}">
+    <comment ref="G2" authorId="0" shapeId="0" xr:uid="{5343DF36-C9C0-470B-A9B1-08DF05F31D2D}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -69,42 +60,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="184">
   <si>
     <t>Veld</t>
   </si>
   <si>
-    <t>Beschrijving voorbeeld</t>
-  </si>
-  <si>
     <t>Beschrijving</t>
   </si>
   <si>
     <t>Conceptbeschrijving</t>
   </si>
   <si>
-    <t>[De definitie of beschrijving van het concept.]</t>
-  </si>
-  <si>
-    <t>PractitionerRole = A specific set of Roles/Locations/specialties/services that a practitioner may perform at an organization for a period of time.</t>
+    <t>Een specifieke samenstelling van (functies/locaties/specialismen/diensten die een zorgverlener kan uitvoeren) bij een organisatie gedurende een bepaalde periode.</t>
   </si>
   <si>
     <t>Doel</t>
   </si>
   <si>
-    <t>[De doelen en redenen om het concept vast te leggen en/of uit te wisselen.]</t>
-  </si>
-  <si>
     <t>Het vastleggen en uitwisselen van gegevens. Primair doel is uitwisseling, secundair doel is vastlegging.</t>
   </si>
   <si>
     <t>Gebruiksscenario(’s)</t>
   </si>
   <si>
-    <t>[Geeft aan in welke context(en) het concept wordt gebruikt. Geef voorbeelden van gebruik in informatiestandaarden.]</t>
-  </si>
-  <si>
-    <t>1. Belangrijk is per dienstverlening aan een patient wie de betrokkenen te weten:
+    <t>Belangrijk is per dienstverlening aan een patient wie de betrokkenen te weten:
 - beroepsrol
 - medische specialisatie
 - persoon
@@ -114,28 +93,16 @@
     <t>Representatie</t>
   </si>
   <si>
-    <t>[Beschrijf hier wat er voor de dossiervorming belangrijk is rondom de levenscyclus en instantiaties van het concept.]</t>
-  </si>
-  <si>
     <t>Het is mogelijk dat de situatie later kan veranderen en daarmee de informatie van het concept</t>
   </si>
   <si>
     <t>Alias(sen)</t>
   </si>
   <si>
-    <t>[Alle bekende synoniemen voor het concept.]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zorgprofessionalrol, Behandelaar, Uitvoerder, Aanvrager, Vaststeller, Verzorger </t>
-  </si>
-  <si>
-    <t>https://hl7.org/fhir/R4/compartmentdefinition-practitioner.html</t>
+    <t>Zorgprofessionalrol, Functiebeschrijving</t>
   </si>
   <si>
     <t>Juist gebruik</t>
-  </si>
-  <si>
-    <t>[Beschrijf hier waarvoor het concept WEL bedoeld is.]</t>
   </si>
   <si>
     <t>1. Om verantwoording aan te geven zodat contact kan worden opgezocht over bepaalde bevindingen
@@ -143,9 +110,6 @@
   </si>
   <si>
     <t>Onjuist gebruik</t>
-  </si>
-  <si>
-    <t>[Beschrijf hier waarvoor het concept NIET bedoeld is.]</t>
   </si>
   <si>
     <r>
@@ -162,7 +126,6 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>natuurlijke persoon die werkzaamheden verricht of gaat verrichten voor een zorgaanbieder en daarbij patiëntgegevens raadpleegt met behulp van een goedgekeurd inlogmiddel</t>
@@ -172,35 +135,25 @@
         <sz val="11"/>
         <color theme="1"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>)</t>
     </r>
   </si>
   <si>
-    <t>Logisch Model</t>
-  </si>
-  <si>
-    <t>[Link naar dataset.]</t>
-  </si>
-  <si>
-    <t>https://decor.nictiz.nl/ad/#/gbb2026bbr-/datasets/dataset/2.16.840.1.113883.2.4.3.11.60.153.1.4/2026-06-08T13:50:54/concept/2.16.840.1.113883.2.4.3.11.60.153.2.1.148/2026-06-08T14:00:05</t>
-  </si>
-  <si>
-    <t>Basis model</t>
-  </si>
-  <si>
-    <t>[Link naar FHIR of OpenEHR model.]</t>
-  </si>
-  <si>
-    <t>https://hl7.org/fhir/R4/practitionerrole.html</t>
+    <t>Referenties</t>
+  </si>
+  <si>
+    <t>zie bronnen tabblad</t>
+  </si>
+  <si>
+    <t>ART-DECOR-id</t>
+  </si>
+  <si>
+    <t>2.16.840.1.113883.2.4.3.11.60.153.4.18/2026-06-11T00:00:00</t>
   </si>
   <si>
     <t>Beredenering basismodel</t>
-  </si>
-  <si>
-    <t>[Beredenering keuze voor basismodel]</t>
   </si>
   <si>
     <t>1. FHIR is het voornaamste internationale data-uitwisselingsmodel
@@ -237,7 +190,7 @@
     <t>FHIR R4 base</t>
   </si>
   <si>
-    <t>https://hl7.org/fhir/R4/practitioner.html</t>
+    <t>https://hl7.org/fhir/R4/practitionerrole.html</t>
   </si>
   <si>
     <t>base FHIR extensions</t>
@@ -249,12 +202,15 @@
     <t>zib-profiel</t>
   </si>
   <si>
-    <t>https://simplifier.net/nictiz-r4-zib2020/~resources?text=healthprofessional&amp;category=Profile</t>
+    <t>https://simplifier.net/nictiz-r4-zib2020/zibhealthprofessionalpractitionerrole</t>
   </si>
   <si>
     <t>NL-core-R4</t>
   </si>
   <si>
+    <t>https://simplifier.net/nictiz-r4-zib2020/nlcorehealthprofessionalpractitionerrole</t>
+  </si>
+  <si>
     <t>EU-core-R4</t>
   </si>
   <si>
@@ -264,7 +220,7 @@
     <t>Xt-EHR LIM</t>
   </si>
   <si>
-    <t>https://www.xt-ehr.eu/fhir/models/0.3.0/StructureDefinition-EHDSHealthProfessional.html</t>
+    <t>https://www.xt-ehr.eu/fhir/models/StructureDefinition-EHDSHealthProfessional.html</t>
   </si>
   <si>
     <t>Xt-EHR LIM --&gt; FHIR mapping</t>
@@ -288,102 +244,243 @@
     <t>Naam</t>
   </si>
   <si>
-    <t>FHIR data-element</t>
-  </si>
-  <si>
     <t>Omschrijving</t>
   </si>
   <si>
     <t>Variabiliteit</t>
   </si>
   <si>
-    <t>Voorwaardelijkheid</t>
+    <t>Aanwezigheid</t>
+  </si>
+  <si>
+    <t>Verleden/heden/toekomst</t>
   </si>
   <si>
     <t>Herkomst</t>
   </si>
   <si>
-    <t>Informatiestandaard</t>
-  </si>
-  <si>
-    <t>Vragen</t>
-  </si>
-  <si>
-    <t>ZVL-004</t>
-  </si>
-  <si>
-    <t>Specialisme</t>
-  </si>
-  <si>
-    <t>PractitionerRole.specialty</t>
+    <t>Opmerkingen</t>
+  </si>
+  <si>
+    <t>ZVR-001</t>
+  </si>
+  <si>
+    <t>Specialisme - PractitionerRole.specialty</t>
   </si>
   <si>
     <t xml:space="preserve">Erkende medische specialismen -&gt;AGB of UZI(DEZI) specialismecodes 
 Het betreft hierbij de erkende medische specialismen zoals vermeld in de wet BIG. Bijvoorbeeld huisarts of cardioloog. </t>
   </si>
   <si>
+    <t xml:space="preserve">coded, AGB en UZI zijn geprefereerde codesystemen voor nederlandse zorgverleners. Binding: Vektis-codelijst </t>
+  </si>
+  <si>
     <t>0..*</t>
   </si>
   <si>
-    <t>AGB en UZI zijn geprefereerde codesystemen voor nederlandse zorgverleners</t>
-  </si>
-  <si>
-    <t>zib2020</t>
-  </si>
-  <si>
-    <t>zib</t>
-  </si>
-  <si>
-    <t>ZVL-005</t>
+    <t>zib2020, Spoedsamenvatting 2.2.0, BgZ-MSZ 2.0</t>
+  </si>
+  <si>
+    <t>ZVR-002</t>
   </si>
   <si>
     <t>Andere codes dan AGB of UZI(DEZI) specialismecodes</t>
   </si>
   <si>
-    <t>Nictiz Sharepoint | Afwijkingenregister eOverdracht</t>
-  </si>
-  <si>
-    <t>e-Overdracht</t>
-  </si>
-  <si>
-    <t>ZVL-008</t>
-  </si>
-  <si>
-    <t>Contactgegevens</t>
-  </si>
-  <si>
-    <t>PractitionerRole.telecom</t>
-  </si>
-  <si>
-    <t>Voor een specifieke rol e.g., werknemer email 
+    <t>(coded) Binding: SNOMED-CT (preferred)</t>
+  </si>
+  <si>
+    <t>EHDSHealthProfessional, Afwijkingenregister eOverdracht</t>
+  </si>
+  <si>
+    <t>ZVR-003</t>
+  </si>
+  <si>
+    <t>Contactgegevens - PractitionerRole.telecom</t>
+  </si>
+  <si>
+    <t>Voor een specifieke rol e.g., werknemer-, locatie-, of specialiteit-email
 Telefoonnummer(s) of e-mailadres(sen), kan ook intercollegiaal telefoonnummer</t>
   </si>
   <si>
-    <t>Niet om te delen; communicatie over de overdracht loopt via Zorgdomein (ZE-1)</t>
-  </si>
-  <si>
-    <t>ZVL-009</t>
-  </si>
-  <si>
-    <t>Zorgaanbieder</t>
-  </si>
-  <si>
-    <t>PractitionerRole.organization</t>
+    <t>(reference GBB-ContactPoint)</t>
+  </si>
+  <si>
+    <t>EHDSHealthProfessional, zib2020, Spoedsamenvatting 2.2.0, BgZ-MSZ 2.0</t>
+  </si>
+  <si>
+    <t>ZVR-004</t>
+  </si>
+  <si>
+    <t>Zorgaanbieder - PractitionerRole.organization</t>
   </si>
   <si>
     <t>Organisatie waarbij de zorgverlener werkzaam is</t>
   </si>
   <si>
+    <t>(reference GBB-Organization)</t>
+  </si>
+  <si>
     <t>0..1</t>
   </si>
   <si>
-    <t>ZVL-012</t>
-  </si>
-  <si>
-    <t>availableTime</t>
-  </si>
-  <si>
-    <t>PractitionerRole.availabletime</t>
+    <t>ZVR-005</t>
+  </si>
+  <si>
+    <t>ProfessionalRole.Role - PractitionerRole.Code</t>
+  </si>
+  <si>
+    <t>Een functietitel zoals verpleegkundige of arts, geen medisch specialisme (bv. Geriatrie) of zorgteamrol (bv. hoofdbehandelaar)
+Binding Description: (preferred): ISCO, SNOMED CT.</t>
+  </si>
+  <si>
+    <t>(coded)</t>
+  </si>
+  <si>
+    <t>EHDSHealthProfessional, Spoedsamenvatting 2.2.0, BgZ-MSZ 2.0</t>
+  </si>
+  <si>
+    <t>ZVR-006</t>
+  </si>
+  <si>
+    <t>Practitioner - verwijzing naar Practitioner profiel</t>
+  </si>
+  <si>
+    <t>Zorgverlener die diensten verleent aan de organisatie</t>
+  </si>
+  <si>
+    <t>(reference GBB-Practitioner)</t>
+  </si>
+  <si>
+    <t>EHDSHealthProfessional, Zib2020 PractitionerRole profiel, Spoedsamenvatting 2.2.0, BgZ-MSZ 2.0</t>
+  </si>
+  <si>
+    <t>ZVR-007</t>
+  </si>
+  <si>
+    <t>TimeInRole</t>
+  </si>
+  <si>
+    <t>Tijdstip of periode waarop de zorgverlener in diens rol was/is</t>
+  </si>
+  <si>
+    <t>periode (start-eindtijden)</t>
+  </si>
+  <si>
+    <t>Spoedsamenvatting 2.2.0</t>
+  </si>
+  <si>
+    <t>Actie</t>
+  </si>
+  <si>
+    <t>Notitie</t>
+  </si>
+  <si>
+    <t>[Actie om te ondernemen, kies uit de 3 acties: cluster, andere bouwsteen en modelleren]</t>
+  </si>
+  <si>
+    <t>[Eventuele notitie]</t>
+  </si>
+  <si>
+    <t>[Naam van de informatie-requirement ]</t>
+  </si>
+  <si>
+    <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
+  </si>
+  <si>
+    <t>[Geef aan wat het element waarmee de informatie-requirement gedekt wordt allemaal zou moeten kunnen. Is het bv. een exacte tijd, en/of een datum, en/of een seizoen?]</t>
+  </si>
+  <si>
+    <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
+  </si>
+  <si>
+    <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
+  </si>
+  <si>
+    <t>Andere bouwsteen</t>
+  </si>
+  <si>
+    <t>Practitioner.identifier</t>
+  </si>
+  <si>
+    <t>Identificatienummer</t>
+  </si>
+  <si>
+    <t>Het zorgverleneridentificatienummer is een nummer dat de zorgverlener uniek identificeert.
+In de Nederlandse situatie worden de volgende nummers gebruikt:
+1. Zorgverlener UZI. Identificatie van zorgverleners (natuurlijke personen) in de Nederlandse zorgsector.
+2. VEKTIS AGB-Z. Dient ter identificatie van zorgverleners en zorgverlenende organisaties
+3. BIG-ID. Het ID van de in het BIG Register opgenomen zorgverlener.
+Voor buitenlandse zorgverleners zijn deze gegevens niet voorhanden.</t>
+  </si>
+  <si>
+    <t>Indien een identificatienummer als UZI of AGB nummer wordt meegegeven, moeten naam en nummer overeenkomen.</t>
+  </si>
+  <si>
+    <t>zib-HealthProfessional-v3.5(2020EN)</t>
+  </si>
+  <si>
+    <t>Cluster</t>
+  </si>
+  <si>
+    <t>Practitioner.name</t>
+  </si>
+  <si>
+    <t>Naamgegevens</t>
+  </si>
+  <si>
+    <t>Practitioner.gender</t>
+  </si>
+  <si>
+    <t>Geslacht</t>
+  </si>
+  <si>
+    <t>Administrative gender</t>
+  </si>
+  <si>
+    <t>Practitioner.address</t>
+  </si>
+  <si>
+    <t>Adresgegevens</t>
+  </si>
+  <si>
+    <t>Van de zorgverlener</t>
+  </si>
+  <si>
+    <t>Wordt soms niet gedeeld wegens privacy, maar kan bereikt worden via Zorgaanbieder</t>
+  </si>
+  <si>
+    <t>Patient.generalPractitioner</t>
+  </si>
+  <si>
+    <t>Zorgverlener(huisarts)</t>
+  </si>
+  <si>
+    <t>"Indien beschikbaar de gegevens van de huisarts van de patiënt"</t>
+  </si>
+  <si>
+    <t>ZorgverlenerRol</t>
+  </si>
+  <si>
+    <t>CareTeam.participant</t>
+  </si>
+  <si>
+    <t>Het concept ZorgverlenerRol kan op twee manieren worden tot uiting worden gebracht, als element in de bouwsteen en als definitiecode bij een verwijzing in een andere bouwsteen (Uitvoerder::Zorgverlener). In beide gevallen wordt voor de code uit dezelfde codelijst geput. Als beide mogelijkheden benut worden, mogen zij niet met elkaar in strijd zijn.</t>
+  </si>
+  <si>
+    <t>Healthprofessional.address (EU-core)</t>
+  </si>
+  <si>
+    <t>PractitionerRole.location</t>
+  </si>
+  <si>
+    <t>(If the address is meant to be where the practitioner provides care.)</t>
+  </si>
+  <si>
+    <t>Opmerking</t>
+  </si>
+  <si>
+    <t>availableTime - PractitionerRole.availabletime</t>
   </si>
   <si>
     <t>Uit zib2020 Contactgegevens.Toelichting (NL-CM:20.6.9) -&gt; "Aangegeven kan bijvoorbeeld worden dat het een afdelingsnummer is (bij zorgverleners) of dat de bereikbaarheid slecht gedurende een aangegeven deel van de dag mogelijk is."</t>
@@ -392,65 +489,34 @@
     <t>https://zibs.nl/wiki/Contactgegevens-v1.2(2020NL)</t>
   </si>
   <si>
-    <t>ZVL-013</t>
-  </si>
-  <si>
-    <t>ProfessionalRole.Role</t>
-  </si>
-  <si>
-    <t>PractitionerRole.Code</t>
-  </si>
-  <si>
-    <t>Health professional role. Multiple roles could be provided.
-Binding Description: (preferred): ISCO, SNOMED CT. De ISCO waardenlijst bevat "occupations" e.g. Nursing professional, Specialist Medical Practitioners.</t>
-  </si>
-  <si>
-    <t>https://build.fhir.org/ig/Xt-EHR/xt-ehr-common/en/StructureDefinition-EHDSHealthProfessional.html</t>
+    <t>Ter Discussie</t>
+  </si>
+  <si>
+    <t>Data element</t>
+  </si>
+  <si>
+    <t>Informatiestandaard</t>
+  </si>
+  <si>
+    <t>Uitleg</t>
+  </si>
+  <si>
+    <t>Uitkomst</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t>Moet DEZI als identifier toegevoegd worden. Niet expliciet genoemd in de zib. Wel al aangekondigd dat het zal worden uitgerold.</t>
+  </si>
+  <si>
+    <t>Wel toegevoegd. In ART-DECOR is er nog geen OID voor. Volgens deze bron wordt gewoon de OID van UZI hergebruikt: https://build.fhir.org/ig/nuts-foundation/nl-generic-functions-ig/credential-DeziUserCredential.html</t>
+  </si>
+  <si>
+    <t>ProfessionalRole</t>
   </si>
   <si>
     <t>EHDSHealthProfessional</t>
-  </si>
-  <si>
-    <t>ZVL-014</t>
-  </si>
-  <si>
-    <t>Practitioner</t>
-  </si>
-  <si>
-    <t>verwijzing naar Practitioner profiel</t>
-  </si>
-  <si>
-    <t>Practitioner that provides services for the organization</t>
-  </si>
-  <si>
-    <t>Zib2020 PractitionerRole profiel</t>
-  </si>
-  <si>
-    <t>ZVL-015</t>
-  </si>
-  <si>
-    <t>Ter Discussie</t>
-  </si>
-  <si>
-    <t>Data element</t>
-  </si>
-  <si>
-    <t>Uitleg</t>
-  </si>
-  <si>
-    <t>Uitkomst</t>
-  </si>
-  <si>
-    <t>Identifier</t>
-  </si>
-  <si>
-    <t>Moet DEZI als identifier toegevoegd worden. Niet expliciet genoemd in de zib. Wel al aangekondigd dat het zal worden uitgerold.</t>
-  </si>
-  <si>
-    <t>Wel toegevoegd. In ART-DECOR is er nog geen OID voor. Volgens deze bron wordt gewoon de OID van UZI hergebruikt: https://build.fhir.org/ig/nuts-foundation/nl-generic-functions-ig/credential-DeziUserCredential.html</t>
-  </si>
-  <si>
-    <t>ProfessionalRole</t>
   </si>
   <si>
     <t>ProfessionalRole bestaat uit role, organization, specialty. Dun onderscheid tussen Role (Multiple roles could be provided.
@@ -458,10 +524,13 @@
 Binding Description: (preferred): SNOMED CT)</t>
   </si>
   <si>
-    <t xml:space="preserve">De ProfessionalRole komt niet overeen met de ZorgverlenerRol(zibs). In NL wordt met Alleen specialty meegenomen in afsprakenmodel. </t>
+    <t xml:space="preserve">De ProfessionalRole komt niet overeen met de ZorgverlenerRol(zibs). Alleen specialty meegenomen in afsprakenmodel. </t>
   </si>
   <si>
     <t>HealthcareProfessionalRoleCodelist</t>
+  </si>
+  <si>
+    <t>zib2020</t>
   </si>
   <si>
     <t>In de zib wordt onder "zorgverlenerrol" verstaan: deelnemer in een zorgteam. Daarom moet deze informatierequirement ondergebracht worden onder het FHIR-profiel "CareTeam"</t>
@@ -479,9 +548,15 @@
     <t>Voor nu erbij gezet (nl.core had het sowieso al), maar een uitleg van de uitsplitsing moet beter worden opgeschreven</t>
   </si>
   <si>
+    <t>availableTime</t>
+  </si>
+  <si>
     <t>Voor nu erbij gezet als string 0..1 (nl.core had het sowieso al), maar alle soorten gebruik van Contactgegevens.Toelichting moeten nog worden uitgestippeld. Ook de invulling van de availableTime in het afsprakenmodel moet nog worden bedacht.</t>
   </si>
   <si>
+    <t>Specialisme</t>
+  </si>
+  <si>
     <t>In NL is het specialisme een UZI of AGB code. In EU is SNOMED preferred.</t>
   </si>
   <si>
@@ -506,6 +581,12 @@
     <t>Telecom</t>
   </si>
   <si>
+    <t>reference(Practitioner)</t>
+  </si>
+  <si>
+    <t>Condition: als AGB/UZI/DEZI, dan reference 1..1</t>
+  </si>
+  <si>
     <t>EN name</t>
   </si>
   <si>
@@ -579,119 +660,6 @@
   </si>
   <si>
     <t>Nu zijn deze allemaal gemapt naar Careteam.participant</t>
-  </si>
-  <si>
-    <t>Actie</t>
-  </si>
-  <si>
-    <t>Notitie</t>
-  </si>
-  <si>
-    <t>Aanwezigheid</t>
-  </si>
-  <si>
-    <t>[Actie om te ondernemen, kies uit de 3 acties: cluster, andere bouwsteen en modelleren]</t>
-  </si>
-  <si>
-    <t>[Eventuele notitie]</t>
-  </si>
-  <si>
-    <t>[Naam van de informatie-requirement ]</t>
-  </si>
-  <si>
-    <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
-  </si>
-  <si>
-    <t>[Geef aan wat het element waarmee de informatie-requirement gedekt wordt allemaal zou moeten kunnen. Is het bv. een exacte tijd, en/of een datum, en/of een seizoen?]</t>
-  </si>
-  <si>
-    <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
-  </si>
-  <si>
-    <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
-  </si>
-  <si>
-    <t>Andere bouwsteen</t>
-  </si>
-  <si>
-    <t>Practitioner.identifier</t>
-  </si>
-  <si>
-    <t>Identificatienummer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Het zorgverleneridentificatienummer is een nummer dat de zorgverlener uniek identificeert.
-In de Nederlandse situatie worden de volgende nummers gebruikt:
-1. Zorgverlener UZI. Identificatie van zorgverleners (natuurlijke personen) in de Nederlandse zorgsector.
-2. VEKTIS AGB-Z. Dient ter identificatie van zorgverleners en zorgverlenende organisaties
-3. BIG-ID. Het ID van de in het BIG Register opgenomen zorgverlener.
-Voor buitenlandse zorgverleners zijn deze gegevens niet voorhanden. </t>
-  </si>
-  <si>
-    <t>Indien een identificatienummer als UZI of AGB nummer wordt meegegeven, moeten naam en nummer overeenkomen.</t>
-  </si>
-  <si>
-    <t>Cluster</t>
-  </si>
-  <si>
-    <t>Practitioner.name</t>
-  </si>
-  <si>
-    <t>Naamgegevens</t>
-  </si>
-  <si>
-    <t>EU-Core</t>
-  </si>
-  <si>
-    <t>Practitioner.gender</t>
-  </si>
-  <si>
-    <t>Geslacht</t>
-  </si>
-  <si>
-    <t>Practitioner.address</t>
-  </si>
-  <si>
-    <t>Adresgegevens</t>
-  </si>
-  <si>
-    <t>Van de zorgverlener</t>
-  </si>
-  <si>
-    <t>Wordt soms niet gedeeld wegens privacy, maar kan bereikt worden via Zorgaanbieder</t>
-  </si>
-  <si>
-    <t>Patient.generalPractitioner</t>
-  </si>
-  <si>
-    <t>Zorgverlener(huisarts)</t>
-  </si>
-  <si>
-    <t>"Indien beschikbaar de gegevens van de huisarts van de patiënt"</t>
-  </si>
-  <si>
-    <t>Kwaliteitsstandaard Uitwisseling Basisgegevensset Zorg tussen instellingen waar medisch-specialistische zorg wordt verleend</t>
-  </si>
-  <si>
-    <t>ZorgverlenerRol</t>
-  </si>
-  <si>
-    <t>CareTeam.participant</t>
-  </si>
-  <si>
-    <t>Het concept ZorgverlenerRol kan op twee manieren worden tot uiting worden gebracht, als element in de bouwsteen en als definitiecode bij een verwijzing in een andere bouwsteen (Uitvoerder::Zorgverlener). In beide gevallen wordt voor de code uit dezelfde codelijst geput. Als beide mogelijkheden benut worden, mogen zij niet met elkaar in strijd zijn.</t>
-  </si>
-  <si>
-    <t>https://www.zibs.nl/images/9/9b/Nl.zorg.Zorgverlener-v3.2%282017NL%29.pdf</t>
-  </si>
-  <si>
-    <t>Healthprofessional.address (EU-core)</t>
-  </si>
-  <si>
-    <t>PractitionerRole.location</t>
-  </si>
-  <si>
-    <t>(If the address is meant to be where the practitioner provides care.)</t>
   </si>
 </sst>
 </file>
@@ -730,49 +698,11 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="2" tint="-0.499984740745262"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="2" tint="-0.499984740745262"/>
-      <name val="Aptos"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos"/>
-      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -788,20 +718,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="2" tint="-0.499984740745262"/>
-      <name val="Aptos"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -842,6 +759,58 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -875,21 +844,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="8">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -940,194 +900,207 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFF1A983"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFF1A983"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFF1A983"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="2" xr:uid="{B0F7F417-6139-AC4A-9919-70BAFABB9069}"/>
   </cellStyles>
-  <dxfs count="30">
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <alignment wrapText="1"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment wrapText="1"/>
-    </dxf>
+  <dxfs count="42">
     <dxf>
       <alignment wrapText="1"/>
     </dxf>
@@ -1206,34 +1179,152 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <fill>
         <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="5" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="10"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <fill>
         <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="5" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
     </dxf>
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
         <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="5" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="5" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -1246,11 +1337,150 @@
       </font>
       <fill>
         <patternFill patternType="none">
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="5" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="5" tint="0.79998168889431442"/>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="5" tint="0.39997558519241921"/>
+        </top>
+        <bottom/>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color theme="5" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top"/>
+    </dxf>
+    <dxf>
+      <font>
+        <u val="none"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1296,11 +1526,7 @@
     </dxf>
     <dxf>
       <font>
-        <b val="0"/>
-        <i val="0"/>
         <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
         <outline val="0"/>
         <shadow val="0"/>
         <u val="none"/>
@@ -1311,6 +1537,12 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -1354,6 +1586,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
+      <alignment horizontal="left" vertical="top"/>
     </dxf>
     <dxf>
       <fill>
@@ -1362,6 +1595,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
+      <alignment horizontal="left" vertical="top"/>
     </dxf>
     <dxf>
       <font>
@@ -1386,7 +1620,7 @@
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1435,6 +1669,45 @@
       </fill>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -1454,6 +1727,154 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>161925</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>223837</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>2181225</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{85C09E76-E7E6-4529-A8D4-95FC581F72B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="163830" y="221932"/>
+          <a:ext cx="6808470" cy="1961198"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Elk concept wordt geïntroduceerd met een tabel die:</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr lvl="0"/>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Het klinische concept identificeert dat door het concept wordt weergegeven, en</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+          </a:br>
+          <a:endParaRPr lang="nl-NL" sz="1100">
+            <a:solidFill>
+              <a:schemeClr val="dk1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:pPr lvl="0"/>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>De belangrijkste kenmerken beschrijft die relevant zijn voor de implementatie, inclusief het beoogde gebruik en veelvoorkomende fouten in gebruik.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="nl-NL" sz="1100">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Deze tabel is bedoeld om een aantal standaard checkvragen te beantwoorden. Deze antwoorden zullen doorgaans blijken uit de informatiebehoefte die onder paragraaf 1.3 beschreven wordt (het is dus niet zo dat eerst de tabel wordt ingevuld en daarna pas de informatiebehoefte).</a:t>
+          </a:r>
+          <a:endParaRPr lang="nl-NL" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -1746,7 +2167,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -1837,72 +2258,97 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C183F3B5-5351-44FE-A16C-8790B0475237}" name="Tabel4" displayName="Tabel4" ref="B2:D12" totalsRowShown="0" headerRowDxfId="29">
-  <autoFilter ref="B2:D12" xr:uid="{C183F3B5-5351-44FE-A16C-8790B0475237}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{4D171181-0874-43D0-941F-6085B024697C}" name="Tabel6" displayName="Tabel6" ref="A2:B12" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+  <autoFilter ref="A2:B12" xr:uid="{4D171181-0874-43D0-941F-6085B024697C}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{B13C53E2-D1C7-49C4-938F-B9875FF88C97}" name="Veld" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{775F1F56-59A2-4007-803C-0EA18F4D6EBF}" name="Beschrijving" dataDxfId="38" dataCellStyle="Hyperlink"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C183F3B5-5351-44FE-A16C-8790B0475237}" name="Tabel4" displayName="Tabel4" ref="A2:C12" totalsRowShown="0" headerRowDxfId="37">
+  <autoFilter ref="A2:C12" xr:uid="{C183F3B5-5351-44FE-A16C-8790B0475237}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{EF90707A-3AD8-4B8C-A5B1-218A9BF91616}" name="type bron" dataDxfId="28"/>
-    <tableColumn id="2" xr3:uid="{3A4760F1-0373-4839-BD85-F34C61857D34}" name="link" dataDxfId="27" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{EF90707A-3AD8-4B8C-A5B1-218A9BF91616}" name="type bron" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{3A4760F1-0373-4839-BD85-F34C61857D34}" name="link" dataDxfId="35" dataCellStyle="Hyperlink"/>
     <tableColumn id="3" xr3:uid="{6FA833D6-F753-4D88-9F39-9DD926E2E2AB}" name="aantekeningen"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="B2:J10" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
-  <autoFilter ref="B2:J10" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
-  <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{A7FC29C7-F2D4-48A5-A359-69D6658FB7BA}" name="FHIR data-element" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Voorwaardelijkheid" dataDxfId="19"/>
-    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Herkomst" dataDxfId="18" dataCellStyle="Hyperlink"/>
-    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Informatiestandaard" dataDxfId="17" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Vragen" dataDxfId="16"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}" name="Tabel362" displayName="Tabel362" ref="B3:E18" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
-  <autoFilter ref="B3:E18" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{2FB2A545-3E03-42E2-A7C5-CBA6BF51E763}" name="Data element" dataDxfId="13"/>
-    <tableColumn id="2" xr3:uid="{B3874943-8B88-43AA-B0A0-4B5081B45198}" name="Informatiestandaard" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{4FFBC5A0-455F-4C81-8A81-963E0DD492F2}" name="Uitleg" dataDxfId="11"/>
-    <tableColumn id="4" xr3:uid="{98900A9D-2F8F-43EC-A740-2203C6F18585}" name="Uitkomst" dataDxfId="10"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="A2:H9" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
+  <autoFilter ref="A2:H9" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="32"/>
+    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="31"/>
+    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="30"/>
+    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="29"/>
+    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Aanwezigheid" dataDxfId="28"/>
+    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Verleden/heden/toekomst" dataDxfId="27" dataCellStyle="Hyperlink"/>
+    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Herkomst" dataDxfId="26" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Opmerkingen" dataDxfId="25"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7CF12276-5DB5-4F90-8695-E8C211C8F244}" name="Tabel5" displayName="Tabel5" ref="A1:G9" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
+  <autoFilter ref="A1:G9" xr:uid="{7CF12276-5DB5-4F90-8695-E8C211C8F244}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{B97F8D91-3082-4CC3-88C3-3AFD25565086}" name="Actie" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{D7C302FA-9136-48F1-8EB1-623FD7B82D0B}" name="Notitie" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{23C47ECA-78A1-46D2-B459-2ED9F0CD69F7}" name="Naam" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{0A87635E-2235-40AA-829B-E1ECCB1E6C33}" name="Omschrijving" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{263135AB-3C6A-4909-9685-2C2C6DED9D81}" name="Variabiliteit" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{698F8C8C-D318-4E44-AD77-5EB91FEF4EFA}" name="Aanwezigheid" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{06FAC50A-4314-452E-8D2E-120AF7C1D687}" name="Herkomst" dataDxfId="16"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{0B8FD523-6F9A-4DD2-B649-F1AB037CCB3E}" name="Tabel7" displayName="Tabel7" ref="A8:F9" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14" tableBorderDxfId="13">
+  <autoFilter ref="A8:F9" xr:uid="{0B8FD523-6F9A-4DD2-B649-F1AB037CCB3E}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{CE30EF06-35A4-4EAF-BCF5-00C597C7326C}" name="Naam" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{947964E3-8FB4-4FA8-9531-0D1655DCB811}" name="Omschrijving" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{C46C9C57-B42E-46EE-A90A-8C42A042008B}" name="Variabiliteit" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{9F619271-6D87-40FC-A84F-CE6461FB1CEF}" name="Aanwezigheid" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{F23BAFE7-FB12-46F9-876F-D325AF2DB821}" name="Herkomst" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{40671050-CB4E-40BA-8D04-BB8D6D9BA49F}" name="Opmerking" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}" name="Tabel362" displayName="Tabel362" ref="B3:E18" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="B3:E18" xr:uid="{F7FDB3CF-22F8-48D8-9133-9B15D32414A7}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{2FB2A545-3E03-42E2-A7C5-CBA6BF51E763}" name="Data element" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{B3874943-8B88-43AA-B0A0-4B5081B45198}" name="Informatiestandaard" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{4FFBC5A0-455F-4C81-8A81-963E0DD492F2}" name="Uitleg" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{98900A9D-2F8F-43EC-A740-2203C6F18585}" name="Uitkomst" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{79DB83F1-8F0F-4AE8-860D-A25F912B5B5C}" name="Tabel3" displayName="Tabel3" ref="B2:E10" totalsRowShown="0">
   <autoFilter ref="B2:E10" xr:uid="{79DB83F1-8F0F-4AE8-860D-A25F912B5B5C}"/>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{E1FF28EC-54D9-4C5E-B216-CE683489BB36}" name="EN name"/>
     <tableColumn id="2" xr3:uid="{9E77889B-1E8C-4DC1-8285-9B73CD19BE32}" name="NL name"/>
     <tableColumn id="3" xr3:uid="{3EC0721C-3350-474C-924F-1C725876433A}" name="FHIR destination"/>
-    <tableColumn id="4" xr3:uid="{47E45A34-8D1A-4889-AE01-49B829C6B42C}" name="Toelichting" dataDxfId="9"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7CF12276-5DB5-4F90-8695-E8C211C8F244}" name="Tabel5" displayName="Tabel5" ref="A1:G7" totalsRowShown="0" headerRowDxfId="8" dataDxfId="7">
-  <autoFilter ref="A1:G7" xr:uid="{7CF12276-5DB5-4F90-8695-E8C211C8F244}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{B97F8D91-3082-4CC3-88C3-3AFD25565086}" name="Actie" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{D7C302FA-9136-48F1-8EB1-623FD7B82D0B}" name="Notitie" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{23C47ECA-78A1-46D2-B459-2ED9F0CD69F7}" name="Naam" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{0A87635E-2235-40AA-829B-E1ECCB1E6C33}" name="Omschrijving" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{263135AB-3C6A-4909-9685-2C2C6DED9D81}" name="Variabiliteit" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{698F8C8C-D318-4E44-AD77-5EB91FEF4EFA}" name="Aanwezigheid" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{06FAC50A-4314-452E-8D2E-120AF7C1D687}" name="Herkomst" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{47E45A34-8D1A-4889-AE01-49B829C6B42C}" name="Toelichting" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2225,318 +2671,293 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="F2" dT="2026-06-10T07:13:12.83" personId="{1324D2D7-870F-4779-B1C5-13BE7166ED9A}" id="{812FD7AE-C33E-4098-9678-0004F1C27ED0}">
-    <text>Vanuit Xt-EHR alleen naamgegevens 0..1, de rest 0..*</text>
-  </threadedComment>
-  <threadedComment ref="I2" dT="2026-06-16T14:38:06.30" personId="{1324D2D7-870F-4779-B1C5-13BE7166ED9A}" id="{5343DF36-C9C0-470B-A9B1-08DF05F31D2D}">
+  <threadedComment ref="G2" dT="2026-06-16T14:38:06.30" personId="{1324D2D7-870F-4779-B1C5-13BE7166ED9A}" id="{5343DF36-C9C0-470B-A9B1-08DF05F31D2D}">
     <text>eOverdracht als basis gebruikt, aanvullend ook zibs2020, zibs2026 en Xt-EHR/EU-Core geraadpleegd</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{44D01FA7-4587-470D-A390-D8587FD365B7}">
-  <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DF696AA-9F2F-43BC-962B-71A16984DFB4}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="40.42578125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="107.28515625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="70.42578125" style="2" customWidth="1"/>
-    <col min="5" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="23" style="33" customWidth="1"/>
+    <col min="2" max="2" width="130" style="33" customWidth="1"/>
+    <col min="3" max="16384" width="9.140625" style="34"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:5" ht="190.5" customHeight="1"/>
+    <row r="2" spans="1:5">
+      <c r="A2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B2" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="12" t="s">
+    </row>
+    <row r="3" spans="1:5" ht="29.25">
+      <c r="A3" s="33" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="29.25">
-      <c r="A2" s="7" t="s">
+      <c r="B3" s="33" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="9" t="s">
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="33" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B4" s="33" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="30">
-      <c r="A3" s="7" t="s">
+      <c r="C4" s="33"/>
+    </row>
+    <row r="5" spans="1:5" ht="78" customHeight="1">
+      <c r="A5" s="33" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="9" t="s">
+      <c r="B5" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C5" s="33"/>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="33" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="87" customHeight="1">
-      <c r="A4" s="7" t="s">
+      <c r="B6" s="36" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C6" s="33"/>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="B7" s="33" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="42.75" customHeight="1">
-      <c r="A5" s="7" t="s">
+      <c r="E7" s="33"/>
+    </row>
+    <row r="8" spans="1:5" ht="29.25">
+      <c r="A8" s="33" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="9" t="s">
+      <c r="B8" s="33" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="E8" s="33"/>
+    </row>
+    <row r="9" spans="1:5" ht="123.75" customHeight="1">
+      <c r="A9" s="33" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="30">
-      <c r="A6" s="7" t="s">
+      <c r="B9" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="C9" s="33"/>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="B10" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="19" t="s">
+      <c r="C10" s="33"/>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="33" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="62.25" customHeight="1">
-      <c r="A7" s="7" t="s">
+      <c r="B11" s="37" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="9" t="s">
+      <c r="C11" s="33"/>
+    </row>
+    <row r="12" spans="1:5" ht="80.25" customHeight="1">
+      <c r="A12" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="B12" s="33" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="138.75" customHeight="1">
-      <c r="A8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="8"/>
-      <c r="B9" s="3"/>
-    </row>
-    <row r="10" spans="1:4" ht="30">
-      <c r="A10" s="7" t="s">
-        <v>25</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C10" s="19" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75">
-      <c r="A11" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C11" s="19" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="75">
-      <c r="A12" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="8"/>
-    </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="8"/>
+      <c r="C12" s="36"/>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="B13" s="38"/>
+      <c r="C13" s="36"/>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="B14" s="38"/>
+      <c r="C14" s="36"/>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="B15" s="38"/>
+      <c r="C15" s="36"/>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="B16" s="38"/>
+      <c r="C16" s="36"/>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" s="38"/>
+      <c r="C17" s="36"/>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" s="38"/>
+      <c r="C18" s="36"/>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" s="38"/>
+      <c r="C19" s="36"/>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" s="38"/>
+      <c r="C20" s="36"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C10" r:id="rId1" location="/gbb2026bbr-/datasets/dataset/2.16.840.1.113883.2.4.3.11.60.153.1.4/2026-06-08T13:50:54/concept/2.16.840.1.113883.2.4.3.11.60.153.2.1.148/2026-06-08T14:00:05" xr:uid="{ED889409-A698-4A14-A40D-FE70B64C7857}"/>
-    <hyperlink ref="C11" r:id="rId2" xr:uid="{A15F1FB0-0D9C-4461-9E1E-58AFB253D7E2}"/>
-    <hyperlink ref="D6" r:id="rId3" xr:uid="{43CF51E7-BFF5-4D03-B360-14A771CE061E}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C04309E7-653D-4B76-B9C4-5CE689010C87}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="87.5703125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="44.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="26.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="87.5703125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="44.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="46"/>
-      <c r="B1" s="46"/>
-      <c r="C1" s="29"/>
-      <c r="D1" s="29"/>
-    </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="28"/>
-      <c r="B2" s="30" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="11"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="13" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C3" s="14"/>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="14"/>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="12"/>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="B7" s="15" t="s">
         <v>35</v>
       </c>
-      <c r="D2" s="30" t="s">
+      <c r="C7" s="14"/>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" s="12" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="28"/>
-      <c r="B3" s="31" t="s">
+      <c r="B8" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="32" t="s">
+      <c r="C8" s="12"/>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="31"/>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29" t="s">
+      <c r="B9" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="C4" s="33" t="s">
+      <c r="C9" s="14"/>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="D4" s="29" t="s">
+      <c r="B10" s="16" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="28"/>
-      <c r="B5" s="31" t="s">
+      <c r="C10" s="12"/>
+    </row>
+    <row r="11" spans="1:3" ht="16.5" customHeight="1">
+      <c r="A11" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="C5" s="32" t="s">
+      <c r="B11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D5" s="31"/>
-    </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="28"/>
-      <c r="B6" s="29" t="s">
+      <c r="C11" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="33" t="s">
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D6" s="29"/>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="28"/>
-      <c r="B7" s="31" t="s">
+      <c r="B12" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="C7" s="32" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="31"/>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="28"/>
-      <c r="B8" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="C8" s="33" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" s="29"/>
-    </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="28"/>
-      <c r="B9" s="31" t="s">
-        <v>49</v>
-      </c>
-      <c r="C9" s="32" t="s">
-        <v>50</v>
-      </c>
-      <c r="D9" s="31"/>
-    </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="28"/>
-      <c r="B10" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="33" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="29"/>
-    </row>
-    <row r="11" spans="1:4" ht="16.5" customHeight="1">
-      <c r="A11" s="28"/>
-      <c r="B11" s="31" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="32" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="34" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="28"/>
-      <c r="B12" s="29" t="s">
-        <v>56</v>
-      </c>
-      <c r="C12" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="D12" s="35"/>
+      <c r="C12" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" xr:uid="{1EAE669F-2594-48D8-B5DD-025264202013}"/>
-    <hyperlink ref="C4" r:id="rId2" xr:uid="{DD0A65EC-3380-449D-9E8D-A8ED17B274E2}"/>
-    <hyperlink ref="C5" r:id="rId3" xr:uid="{AFABA083-6D7B-42D6-A2F8-DEBF63ECFDB2}"/>
-    <hyperlink ref="C6" r:id="rId4" xr:uid="{63F21764-18AB-425F-9D40-4CAC7C7C1493}"/>
-    <hyperlink ref="C7" r:id="rId5" xr:uid="{B1F18E64-7EF6-4E4D-9B32-A47DC8115924}"/>
-    <hyperlink ref="C8" r:id="rId6" xr:uid="{2370A320-2121-4D79-BC3A-54A3C11EB1EA}"/>
-    <hyperlink ref="C9" r:id="rId7" xr:uid="{EF4942F1-8231-4290-9C58-C9837013E0F3}"/>
-    <hyperlink ref="C10" r:id="rId8" xr:uid="{34D09E24-B386-407B-9332-93B9974AC3C5}"/>
-    <hyperlink ref="C11" r:id="rId9" xr:uid="{28B1F381-AC28-4874-9868-14509FD24CDE}"/>
-    <hyperlink ref="C12" r:id="rId10" xr:uid="{C6A0DAFE-5CCB-47CE-83B4-463EB7BB2F08}"/>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{1EAE669F-2594-48D8-B5DD-025264202013}"/>
+    <hyperlink ref="B4" r:id="rId2" xr:uid="{DD0A65EC-3380-449D-9E8D-A8ED17B274E2}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{AFABA083-6D7B-42D6-A2F8-DEBF63ECFDB2}"/>
+    <hyperlink ref="B6" r:id="rId4" xr:uid="{63F21764-18AB-425F-9D40-4CAC7C7C1493}"/>
+    <hyperlink ref="B7" r:id="rId5" xr:uid="{B1F18E64-7EF6-4E4D-9B32-A47DC8115924}"/>
+    <hyperlink ref="B8" r:id="rId6" xr:uid="{2370A320-2121-4D79-BC3A-54A3C11EB1EA}"/>
+    <hyperlink ref="B9" r:id="rId7" xr:uid="{EF4942F1-8231-4290-9C58-C9837013E0F3}"/>
+    <hyperlink ref="B10" r:id="rId8" xr:uid="{34D09E24-B386-407B-9332-93B9974AC3C5}"/>
+    <hyperlink ref="B11" r:id="rId9" xr:uid="{28B1F381-AC28-4874-9868-14509FD24CDE}"/>
+    <hyperlink ref="B12" r:id="rId10" xr:uid="{C6A0DAFE-5CCB-47CE-83B4-463EB7BB2F08}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -2547,440 +2968,700 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C1A0E3D-BE28-4965-A5FF-C835B3665CFB}">
-  <dimension ref="B2:L10"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A2:J13"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="31" customWidth="1"/>
-    <col min="5" max="6" width="65.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="82.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="37.7109375" customWidth="1"/>
-    <col min="9" max="9" width="15.7109375" customWidth="1"/>
-    <col min="10" max="10" width="35.28515625" customWidth="1"/>
-    <col min="11" max="11" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.42578125" style="41" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31" style="41" customWidth="1"/>
+    <col min="3" max="3" width="69.7109375" style="47" customWidth="1"/>
+    <col min="4" max="4" width="31.7109375" style="47" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" style="47" customWidth="1"/>
+    <col min="6" max="6" width="37.7109375" style="41" customWidth="1"/>
+    <col min="7" max="7" width="23.140625" style="41" customWidth="1"/>
+    <col min="8" max="8" width="35.28515625" style="41" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" style="41" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="41"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" ht="30">
-      <c r="B2" s="17" t="s">
+    <row r="2" spans="1:10">
+      <c r="A2" s="39" t="s">
+        <v>47</v>
+      </c>
+      <c r="B2" s="40" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="I2" s="40"/>
+      <c r="J2" s="40"/>
+    </row>
+    <row r="3" spans="1:10" s="45" customFormat="1" ht="57.75">
+      <c r="A3" s="42" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="C3" s="43" t="s">
+        <v>57</v>
+      </c>
+      <c r="D3" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="E3" s="43" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F3" s="31"/>
+      <c r="G3" s="32" t="s">
         <v>60</v>
       </c>
-      <c r="E2" s="5" t="s">
+    </row>
+    <row r="4" spans="1:10" ht="43.5">
+      <c r="A4" s="42" t="s">
         <v>61</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="B4" s="43" t="s">
+        <v>56</v>
+      </c>
+      <c r="C4" s="43" t="s">
         <v>62</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="D4" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="E4" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" s="31"/>
+      <c r="G4" s="32" t="s">
         <v>64</v>
       </c>
-      <c r="I2" s="5" t="s">
+    </row>
+    <row r="5" spans="1:10" s="45" customFormat="1" ht="57.75">
+      <c r="A5" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="B5" s="43" t="s">
         <v>66</v>
       </c>
-      <c r="K2" s="5"/>
-      <c r="L2" s="5"/>
-    </row>
-    <row r="3" spans="2:12" s="23" customFormat="1" ht="43.5">
-      <c r="B3" s="14" t="s">
+      <c r="C5" s="43" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="D5" s="46" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="E5" s="43" t="s">
+        <v>59</v>
+      </c>
+      <c r="F5" s="31"/>
+      <c r="G5" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="E3" s="10" t="s">
+    </row>
+    <row r="6" spans="1:10" s="45" customFormat="1" ht="57.75">
+      <c r="A6" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="B6" s="43" t="s">
         <v>71</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="C6" s="43" t="s">
         <v>72</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="D6" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="I3" s="10" t="s">
+      <c r="E6" s="43" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="4" spans="2:12" ht="29.25">
-      <c r="B4" s="14" t="s">
+      <c r="F6" s="31"/>
+      <c r="G6" s="32" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="48" customFormat="1" ht="68.25" customHeight="1">
+      <c r="A7" s="42" t="s">
         <v>75</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="E4" s="10" t="s">
+      <c r="B7" s="46" t="s">
         <v>76</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="H4" s="22" t="s">
+      <c r="C7" s="46" t="s">
         <v>77</v>
       </c>
-      <c r="I4" s="10" t="s">
+      <c r="D7" s="46" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="5" spans="2:12" s="23" customFormat="1" ht="43.5">
-      <c r="B5" s="14" t="s">
+      <c r="E7" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="F7" s="31"/>
+      <c r="G7" s="47" t="s">
         <v>79</v>
       </c>
-      <c r="C5" s="10" t="s">
+    </row>
+    <row r="8" spans="1:10" s="48" customFormat="1" ht="72.75">
+      <c r="A8" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="B8" s="46" t="s">
         <v>81</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="C8" s="41" t="s">
         <v>82</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G5" s="21" t="s">
+      <c r="D8" s="46" t="s">
         <v>83</v>
       </c>
-      <c r="H5" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="I5" s="10"/>
-    </row>
-    <row r="6" spans="2:12" s="23" customFormat="1">
-      <c r="B6" s="14" t="s">
+      <c r="E8" s="46" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="31"/>
+      <c r="G8" s="32" t="s">
         <v>84</v>
       </c>
-      <c r="C6" s="10" t="s">
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="B9" s="46" t="s">
         <v>86</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="C9" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="D9" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="G6" s="21"/>
-      <c r="H6" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="I6" s="10"/>
-    </row>
-    <row r="7" spans="2:12" s="26" customFormat="1" ht="57.75">
-      <c r="B7" s="14" t="s">
+      <c r="E9" s="46" t="s">
+        <v>74</v>
+      </c>
+      <c r="F9" s="31"/>
+      <c r="G9" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="C7" s="13" t="s">
+    </row>
+    <row r="12" spans="1:10">
+      <c r="E12" s="41"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="E13" s="41"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{688495E5-0C43-4F64-B944-96A9F5BA516C}">
+  <dimension ref="A1:H11"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="19" style="1" customWidth="1"/>
+    <col min="2" max="2" width="39" style="1" customWidth="1"/>
+    <col min="3" max="3" width="33" style="1" customWidth="1"/>
+    <col min="4" max="4" width="81.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="14.42578125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="54.7109375" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="168.75" customHeight="1">
+      <c r="A1" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="B1" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="C1" s="19" t="s">
+        <v>48</v>
+      </c>
+      <c r="D1" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="E1" s="19" t="s">
+        <v>50</v>
+      </c>
+      <c r="F1" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" s="19" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="188.45" hidden="1">
+      <c r="A2" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="F7" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="G7" s="25"/>
-      <c r="H7" s="16" t="s">
+      <c r="B2" s="20" t="s">
         <v>93</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="C2" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="F2" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="116.1">
+      <c r="A3" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="G3" s="30" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="8" spans="2:12" s="26" customFormat="1" ht="57.75">
-      <c r="B8" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>95</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>96</v>
-      </c>
-      <c r="E8" s="13" t="s">
-        <v>97</v>
-      </c>
-      <c r="F8" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="G8" s="25"/>
-      <c r="H8" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="I8" s="16" t="s">
+      <c r="G4" s="30" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="1" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="9" spans="2:12" s="26" customFormat="1">
-      <c r="B9" s="14" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="E9" t="s">
-        <v>103</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="G9" s="25"/>
-      <c r="H9" s="16" t="s">
+      <c r="B5" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="30" t="s">
         <v>104</v>
       </c>
-      <c r="I9" s="16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="10" spans="2:12">
-      <c r="B10" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="25"/>
-      <c r="H10" s="16"/>
-      <c r="I10" s="16"/>
+    </row>
+    <row r="6" spans="1:8" ht="29.1">
+      <c r="A6" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G6" s="30" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="G7" s="30" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" s="8" customFormat="1" ht="66.75" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F8" s="7"/>
+      <c r="G8" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="H8" s="3"/>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="28" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="C9" s="28" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="29" t="s">
+        <v>123</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="30" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="C11"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="12" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="H7" r:id="rId1" xr:uid="{FEB7522F-2A9D-49C2-82F5-222BEE2F9415}"/>
-    <hyperlink ref="H8" r:id="rId2" xr:uid="{708A4C80-C2CD-48E7-8282-4E696A81C206}"/>
+    <hyperlink ref="G3" r:id="rId1" xr:uid="{73B0A1AA-23A8-4A3C-8630-433382D48C85}"/>
+    <hyperlink ref="G4:G9" r:id="rId2" display="zib-HealthProfessional-v3.5(2020EN)" xr:uid="{993879EF-A105-4DD4-A73F-C6E1351F1F56}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId3"/>
+  <drawing r:id="rId3"/>
   <tableParts count="1">
     <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8748DCD5-A959-41F5-9A2D-B277CB3E46A1}">
+  <dimension ref="A8:G9"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="21.85546875" style="49" customWidth="1"/>
+    <col min="2" max="2" width="66.28515625" style="49" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="49" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" style="49" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" style="49" customWidth="1"/>
+    <col min="6" max="7" width="10.28515625" style="49" bestFit="1" customWidth="1"/>
+    <col min="8" max="16384" width="9.140625" style="49"/>
+  </cols>
+  <sheetData>
+    <row r="8" spans="1:7">
+      <c r="A8" s="49" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" s="49" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="49" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" s="49" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="49" t="s">
+        <v>53</v>
+      </c>
+      <c r="F8" s="49" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="87">
+      <c r="A9" s="50" t="s">
+        <v>125</v>
+      </c>
+      <c r="B9" s="50" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>59</v>
+      </c>
+      <c r="D9" s="52"/>
+      <c r="E9" s="53" t="s">
+        <v>127</v>
+      </c>
+      <c r="F9" s="54"/>
+      <c r="G9" s="55"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E9" r:id="rId1" xr:uid="{FEB7522F-2A9D-49C2-82F5-222BEE2F9415}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId2"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B1E71E66-FD43-4603-91A3-4CCDD6133986}">
   <dimension ref="B2:H24"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="3.85546875" style="4" customWidth="1"/>
-    <col min="2" max="2" width="21.42578125" style="4" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" style="4" customWidth="1"/>
-    <col min="4" max="4" width="74" style="4" customWidth="1"/>
-    <col min="5" max="5" width="65.28515625" style="4" customWidth="1"/>
-    <col min="6" max="6" width="24.42578125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="21.7109375" style="4" customWidth="1"/>
-    <col min="8" max="8" width="73.7109375" style="4" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="4"/>
+    <col min="1" max="1" width="3.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="21.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="74" style="2" customWidth="1"/>
+    <col min="5" max="5" width="65.28515625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="24.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="21.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="73.7109375" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8">
-      <c r="B2" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="F2" s="27"/>
+      <c r="B2" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="F2" s="10"/>
     </row>
     <row r="3" spans="2:8">
-      <c r="B3" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="D3" s="15" t="s">
-        <v>108</v>
-      </c>
-      <c r="E3" s="24" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-    </row>
-    <row r="4" spans="2:8" ht="60">
-      <c r="B4" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="5" spans="2:8" ht="78" customHeight="1">
-      <c r="B5" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>114</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="6" spans="2:8" ht="45">
-      <c r="B6" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" ht="75">
-      <c r="B7" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>119</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="8" spans="2:8" ht="57.75">
-      <c r="B8" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>92</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>121</v>
+      <c r="B3" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" spans="2:8" ht="43.5">
+      <c r="B4" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="102.75" customHeight="1">
+      <c r="B5" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="6" spans="2:8" ht="43.5">
+      <c r="B6" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="105.75" customHeight="1">
+      <c r="B7" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" ht="64.5" customHeight="1">
+      <c r="B8" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="9" spans="2:8">
-      <c r="B9" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>122</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>123</v>
+      <c r="B9" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="10" spans="2:8">
-      <c r="B10" s="4" t="s">
-        <v>124</v>
+      <c r="B10" s="2" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="11" spans="2:8">
-      <c r="B11" s="41" t="s">
-        <v>125</v>
-      </c>
-      <c r="C11" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="42" t="s">
-        <v>126</v>
-      </c>
-      <c r="E11" s="43" t="s">
-        <v>127</v>
+      <c r="B11" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="2:8">
-      <c r="B12" s="44" t="s">
-        <v>128</v>
-      </c>
-      <c r="C12" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="45" t="s">
-        <v>126</v>
-      </c>
-      <c r="E12" s="40" t="s">
-        <v>127</v>
+      <c r="B12" s="25" t="s">
+        <v>155</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="E12" s="21" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="2:8">
-      <c r="B13" s="41" t="s">
-        <v>110</v>
-      </c>
-      <c r="C13" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13" s="42" t="s">
-        <v>126</v>
-      </c>
-      <c r="E13" s="43" t="s">
-        <v>127</v>
+      <c r="B13" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="C13" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D13" s="23" t="s">
+        <v>153</v>
+      </c>
+      <c r="E13" s="24" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="2:8">
-      <c r="B14" s="44" t="s">
-        <v>129</v>
-      </c>
-      <c r="C14" s="42" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14" s="45" t="s">
-        <v>126</v>
-      </c>
-      <c r="E14" s="40" t="s">
-        <v>127</v>
+      <c r="B14" s="25" t="s">
+        <v>156</v>
+      </c>
+      <c r="C14" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="E14" s="21" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="15" spans="2:8" ht="15">
+      <c r="B15" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="2:4">
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
     </row>
     <row r="19" spans="2:4" ht="19.5" customHeight="1">
-      <c r="B19" s="13"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="13"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
     </row>
     <row r="20" spans="2:4" ht="19.5" customHeight="1">
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="13"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
     </row>
     <row r="21" spans="2:4" ht="19.5" customHeight="1"/>
     <row r="24" spans="2:4">
-      <c r="B24" s="20"/>
-      <c r="C24" s="20"/>
-      <c r="D24" s="20"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2990,10 +3671,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D7E96EB-0EDF-43CA-9149-BA391692EDD0}">
   <dimension ref="B2:E12"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="2" max="2" width="22.7109375" customWidth="1"/>
     <col min="3" max="3" width="27.42578125" customWidth="1"/>
@@ -3003,109 +3684,109 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" t="s">
-        <v>130</v>
+        <v>159</v>
       </c>
       <c r="C2" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="D2" t="s">
-        <v>132</v>
+        <v>161</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>133</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
       <c r="C3" t="s">
-        <v>135</v>
+        <v>164</v>
       </c>
       <c r="D3" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" t="s">
-        <v>137</v>
+        <v>166</v>
       </c>
       <c r="C4" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="5" spans="2:5" ht="45">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="5" spans="2:5" ht="43.5">
       <c r="B5" t="s">
-        <v>139</v>
+        <v>168</v>
       </c>
       <c r="C5" t="s">
-        <v>140</v>
+        <v>169</v>
       </c>
       <c r="D5" t="s">
-        <v>141</v>
+        <v>170</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>142</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" t="s">
-        <v>143</v>
+        <v>172</v>
       </c>
       <c r="C6" t="s">
-        <v>144</v>
+        <v>173</v>
       </c>
       <c r="D6" t="s">
-        <v>145</v>
+        <v>174</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>145</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" t="s">
-        <v>146</v>
+        <v>175</v>
       </c>
       <c r="C7" t="s">
-        <v>147</v>
+        <v>176</v>
       </c>
       <c r="D7" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="8" spans="2:5" ht="45">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="8" spans="2:5" ht="43.5">
       <c r="B8" t="s">
-        <v>148</v>
+        <v>177</v>
       </c>
       <c r="C8" t="s">
-        <v>149</v>
+        <v>178</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>150</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="B9" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="C9" t="s">
-        <v>151</v>
+        <v>180</v>
       </c>
       <c r="D9" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" t="s">
-        <v>152</v>
+        <v>181</v>
       </c>
       <c r="C10" t="s">
-        <v>153</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="2:5">
-      <c r="B12" t="s">
-        <v>154</v>
+      <c r="B12" s="27" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -3113,214 +3794,6 @@
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{688495E5-0C43-4F64-B944-96A9F5BA516C}">
-  <dimension ref="A1:H11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="19" style="1" customWidth="1"/>
-    <col min="2" max="4" width="54.7109375" style="1" customWidth="1"/>
-    <col min="5" max="5" width="22" style="1" customWidth="1"/>
-    <col min="6" max="7" width="54.7109375" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" ht="168.75" customHeight="1">
-      <c r="A1" s="36" t="s">
-        <v>155</v>
-      </c>
-      <c r="B1" s="36" t="s">
-        <v>156</v>
-      </c>
-      <c r="C1" s="36" t="s">
-        <v>59</v>
-      </c>
-      <c r="D1" s="36" t="s">
-        <v>61</v>
-      </c>
-      <c r="E1" s="36" t="s">
-        <v>62</v>
-      </c>
-      <c r="F1" s="36" t="s">
-        <v>157</v>
-      </c>
-      <c r="G1" s="36" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" ht="115.5" hidden="1">
-      <c r="A2" s="37" t="s">
-        <v>158</v>
-      </c>
-      <c r="B2" s="37" t="s">
-        <v>159</v>
-      </c>
-      <c r="C2" s="37" t="s">
-        <v>160</v>
-      </c>
-      <c r="D2" s="37" t="s">
-        <v>161</v>
-      </c>
-      <c r="E2" s="37" t="s">
-        <v>162</v>
-      </c>
-      <c r="F2" s="37" t="s">
-        <v>163</v>
-      </c>
-      <c r="G2" s="37" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" ht="212.25" customHeight="1">
-      <c r="A3" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="1" t="s">
-        <v>170</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" ht="29.25">
-      <c r="A6" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>178</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="29.25">
-      <c r="A7" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>180</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>181</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>182</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" s="23" customFormat="1" ht="87">
-      <c r="A8" s="38" t="s">
-        <v>165</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>184</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>185</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>186</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>71</v>
-      </c>
-      <c r="F8" s="21"/>
-      <c r="G8" s="22" t="s">
-        <v>187</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="29.25">
-      <c r="A9" s="39" t="s">
-        <v>165</v>
-      </c>
-      <c r="B9" s="39" t="s">
-        <v>188</v>
-      </c>
-      <c r="C9" s="39" t="s">
-        <v>189</v>
-      </c>
-      <c r="D9" s="40" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="C11"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <tableParts count="1">
-    <tablePart r:id="rId2"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8748DCD5-A959-41F5-9A2D-B277CB3E46A1}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
PractitionerRole: added EU filter row
</commit_message>
<xml_diff>
--- a/input/requirements/PractitionerRole.xlsx
+++ b/input/requirements/PractitionerRole.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/PractitionerRole/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3045" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4D37651-9E16-4768-8594-450EB93BF6B1}"/>
+  <xr:revisionPtr revIDLastSave="3046" documentId="8_{E18A75D0-0588-41D5-84D2-F29C11C8C8B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E05AC87B-58A3-4EC7-AEF2-3BCE14A297A5}"/>
   <bookViews>
-    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" tabRatio="655" firstSheet="2" activeTab="6" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" tabRatio="655" firstSheet="6" activeTab="6" xr2:uid="{46BF2C1A-54CB-44AC-9917-BC7A0C964166}"/>
   </bookViews>
   <sheets>
     <sheet name="Concept" sheetId="18" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="239" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="185">
   <si>
     <t>Veld</t>
   </si>
@@ -260,6 +260,9 @@
   </si>
   <si>
     <t>Opmerkingen</t>
+  </si>
+  <si>
+    <t>EU filter</t>
   </si>
   <si>
     <t>ZVR-001</t>
@@ -939,7 +942,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1047,60 +1050,59 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
     <cellStyle name="Standaard 2" xfId="2" xr:uid="{B0F7F417-6139-AC4A-9919-70BAFABB9069}"/>
   </cellStyles>
-  <dxfs count="42">
+  <dxfs count="43">
     <dxf>
       <alignment wrapText="1"/>
     </dxf>
@@ -1447,6 +1449,16 @@
         <scheme val="minor"/>
       </font>
       <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top"/>
     </dxf>
     <dxf>
       <fill>
@@ -2258,22 +2270,22 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{4D171181-0874-43D0-941F-6085B024697C}" name="Tabel6" displayName="Tabel6" ref="A2:B12" totalsRowShown="0" headerRowDxfId="41" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{4D171181-0874-43D0-941F-6085B024697C}" name="Tabel6" displayName="Tabel6" ref="A2:B12" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
   <autoFilter ref="A2:B12" xr:uid="{4D171181-0874-43D0-941F-6085B024697C}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{B13C53E2-D1C7-49C4-938F-B9875FF88C97}" name="Veld" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{775F1F56-59A2-4007-803C-0EA18F4D6EBF}" name="Beschrijving" dataDxfId="38" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{B13C53E2-D1C7-49C4-938F-B9875FF88C97}" name="Veld" dataDxfId="40"/>
+    <tableColumn id="2" xr3:uid="{775F1F56-59A2-4007-803C-0EA18F4D6EBF}" name="Beschrijving" dataDxfId="39" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C183F3B5-5351-44FE-A16C-8790B0475237}" name="Tabel4" displayName="Tabel4" ref="A2:C12" totalsRowShown="0" headerRowDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{C183F3B5-5351-44FE-A16C-8790B0475237}" name="Tabel4" displayName="Tabel4" ref="A2:C12" totalsRowShown="0" headerRowDxfId="38">
   <autoFilter ref="A2:C12" xr:uid="{C183F3B5-5351-44FE-A16C-8790B0475237}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{EF90707A-3AD8-4B8C-A5B1-218A9BF91616}" name="type bron" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{3A4760F1-0373-4839-BD85-F34C61857D34}" name="link" dataDxfId="35" dataCellStyle="Hyperlink"/>
+    <tableColumn id="1" xr3:uid="{EF90707A-3AD8-4B8C-A5B1-218A9BF91616}" name="type bron" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{3A4760F1-0373-4839-BD85-F34C61857D34}" name="link" dataDxfId="36" dataCellStyle="Hyperlink"/>
     <tableColumn id="3" xr3:uid="{6FA833D6-F753-4D88-9F39-9DD926E2E2AB}" name="aantekeningen"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2281,17 +2293,20 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="A2:H9" totalsRowShown="0" headerRowDxfId="34" dataDxfId="33">
-  <autoFilter ref="A2:H9" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="32"/>
-    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="31"/>
-    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="30"/>
-    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="29"/>
-    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Aanwezigheid" dataDxfId="28"/>
-    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Verleden/heden/toekomst" dataDxfId="27" dataCellStyle="Hyperlink"/>
-    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Herkomst" dataDxfId="26" dataCellStyle="Hyperlink"/>
-    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Opmerkingen" dataDxfId="25"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}" name="Tabel1" displayName="Tabel1" ref="A2:I9" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+  <autoFilter ref="A2:I9" xr:uid="{46AECDBA-D052-4545-915C-E549FBECFE2B}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{FEE75A6E-51DE-4226-8B24-56203341A5FB}" name="Nummer" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{C6ED2961-D275-431D-B06A-13A385D01FD7}" name="Naam" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{800A371F-5934-43D8-B1D5-B68739655D17}" name="Omschrijving" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{36532627-584F-4D2E-950B-CBC991B0B85D}" name="Variabiliteit" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{F05C3C30-E136-4C9E-B547-3FB89A6146FE}" name="Aanwezigheid" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{6B2B916E-EB05-4FD4-9722-3E3F9CFF1689}" name="Verleden/heden/toekomst" dataDxfId="28" dataCellStyle="Hyperlink"/>
+    <tableColumn id="8" xr3:uid="{7066775C-D7C5-4494-A3A0-C56203FC7E6E}" name="Herkomst" dataDxfId="27" dataCellStyle="Hyperlink"/>
+    <tableColumn id="7" xr3:uid="{683B86F6-FA23-479B-BB80-9E4FB1070E15}" name="Opmerkingen" dataDxfId="26"/>
+    <tableColumn id="9" xr3:uid="{02778FF9-3916-4097-BB73-F7ED357F0808}" name="EU filter" dataDxfId="25">
+      <calculatedColumnFormula>ISNUMBER(SEARCH("EHDS", G3))</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2971,198 +2986,228 @@
   <dimension ref="A2:J13"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" style="41" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31" style="41" customWidth="1"/>
-    <col min="3" max="3" width="69.7109375" style="47" customWidth="1"/>
-    <col min="4" max="4" width="31.7109375" style="47" customWidth="1"/>
-    <col min="5" max="5" width="18.7109375" style="47" customWidth="1"/>
-    <col min="6" max="6" width="37.7109375" style="41" customWidth="1"/>
-    <col min="7" max="7" width="23.140625" style="41" customWidth="1"/>
-    <col min="8" max="8" width="35.28515625" style="41" customWidth="1"/>
-    <col min="9" max="9" width="8.85546875" style="41" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="41"/>
+    <col min="1" max="1" width="10.42578125" style="40" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="31" style="40" customWidth="1"/>
+    <col min="3" max="3" width="69.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="31.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="18.7109375" style="2" customWidth="1"/>
+    <col min="6" max="6" width="37.7109375" style="40" customWidth="1"/>
+    <col min="7" max="7" width="23.140625" style="40" customWidth="1"/>
+    <col min="8" max="8" width="35.28515625" style="40" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" style="40" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.85546875" style="40"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:10">
       <c r="A2" s="39" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="40" t="s">
+      <c r="B2" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C2" s="40" t="s">
+      <c r="C2" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="40" t="s">
+      <c r="D2" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="40" t="s">
+      <c r="E2" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="40" t="s">
+      <c r="F2" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="G2" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="H2" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="40"/>
-      <c r="J2" s="40"/>
-    </row>
-    <row r="3" spans="1:10" s="45" customFormat="1" ht="57.75">
-      <c r="A3" s="42" t="s">
+      <c r="I2" s="54" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="J2" s="6"/>
+    </row>
+    <row r="3" spans="1:10" s="43" customFormat="1" ht="57.75">
+      <c r="A3" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="43" t="s">
+      <c r="B3" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="D3" s="44" t="s">
+      <c r="C3" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="E3" s="43" t="s">
+      <c r="D3" s="42" t="s">
         <v>59</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="F3" s="31"/>
       <c r="G3" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="I3" s="50" t="b">
+        <f t="shared" ref="I3:I9" si="0">ISNUMBER(SEARCH("EHDS", G3))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="43.5">
+      <c r="A4" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" s="3" t="s">
         <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="43.5">
-      <c r="A4" s="42" t="s">
-        <v>61</v>
-      </c>
-      <c r="B4" s="43" t="s">
-        <v>56</v>
-      </c>
-      <c r="C4" s="43" t="s">
-        <v>62</v>
-      </c>
-      <c r="D4" s="46" t="s">
-        <v>63</v>
-      </c>
-      <c r="E4" s="43" t="s">
-        <v>59</v>
       </c>
       <c r="F4" s="31"/>
       <c r="G4" s="32" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" s="45" customFormat="1" ht="57.75">
-      <c r="A5" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="B5" s="43" t="s">
+      <c r="I4" s="50" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="43" customFormat="1" ht="57.75">
+      <c r="A5" s="41" t="s">
         <v>66</v>
       </c>
-      <c r="C5" s="43" t="s">
+      <c r="B5" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D5" s="46" t="s">
+      <c r="C5" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E5" s="43" t="s">
-        <v>59</v>
+      <c r="D5" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>60</v>
       </c>
       <c r="F5" s="31"/>
       <c r="G5" s="32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" s="45" customFormat="1" ht="57.75">
-      <c r="A6" s="42" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="43" t="s">
+      <c r="I5" s="51" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" s="43" customFormat="1" ht="57.75">
+      <c r="A6" s="41" t="s">
         <v>71</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="B6" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="D6" s="46" t="s">
+      <c r="C6" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="E6" s="43" t="s">
+      <c r="D6" s="4" t="s">
         <v>74</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>75</v>
       </c>
       <c r="F6" s="31"/>
       <c r="G6" s="32" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" s="48" customFormat="1" ht="68.25" customHeight="1">
-      <c r="A7" s="42" t="s">
+        <v>70</v>
+      </c>
+      <c r="I6" s="51" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" s="44" customFormat="1" ht="68.25" customHeight="1">
+      <c r="A7" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="31"/>
+      <c r="G7" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="I7" s="52" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" s="44" customFormat="1" ht="72.75">
+      <c r="A8" s="41" t="s">
+        <v>81</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C8" s="40" t="s">
+        <v>83</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>75</v>
-      </c>
-      <c r="B7" s="46" t="s">
-        <v>76</v>
-      </c>
-      <c r="C7" s="46" t="s">
-        <v>77</v>
-      </c>
-      <c r="D7" s="46" t="s">
-        <v>78</v>
-      </c>
-      <c r="E7" s="46" t="s">
-        <v>59</v>
-      </c>
-      <c r="F7" s="31"/>
-      <c r="G7" s="47" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" s="48" customFormat="1" ht="72.75">
-      <c r="A8" s="42" t="s">
-        <v>80</v>
-      </c>
-      <c r="B8" s="46" t="s">
-        <v>81</v>
-      </c>
-      <c r="C8" s="41" t="s">
-        <v>82</v>
-      </c>
-      <c r="D8" s="46" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="46" t="s">
-        <v>74</v>
       </c>
       <c r="F8" s="31"/>
       <c r="G8" s="32" t="s">
-        <v>84</v>
+        <v>85</v>
+      </c>
+      <c r="I8" s="52" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="42" t="s">
-        <v>85</v>
-      </c>
-      <c r="B9" s="46" t="s">
+      <c r="A9" s="41" t="s">
         <v>86</v>
       </c>
-      <c r="C9" s="46" t="s">
+      <c r="B9" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D9" s="46" t="s">
+      <c r="C9" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E9" s="46" t="s">
-        <v>74</v>
+      <c r="D9" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>75</v>
       </c>
       <c r="F9" s="31"/>
       <c r="G9" s="32" t="s">
-        <v>89</v>
+        <v>90</v>
+      </c>
+      <c r="I9" s="53" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:10">
-      <c r="E12" s="41"/>
+      <c r="E12" s="40"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="E13" s="41"/>
+      <c r="E13" s="40"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
@@ -3189,10 +3234,10 @@
   <sheetData>
     <row r="1" spans="1:8" ht="168.75" customHeight="1">
       <c r="A1" s="19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B1" s="19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C1" s="19" t="s">
         <v>48</v>
@@ -3212,170 +3257,170 @@
     </row>
     <row r="2" spans="1:8" ht="188.45" hidden="1">
       <c r="A2" s="20" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C2" s="20" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D2" s="20" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F2" s="20" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G2" s="20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="116.1">
       <c r="A3" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G3" s="30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="G4" s="30" t="s">
         <v>105</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="G4" s="30" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G5" s="30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="29.1">
       <c r="A6" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G6" s="30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G7" s="30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:8" s="8" customFormat="1" ht="66.75" customHeight="1">
       <c r="A8" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8" s="7"/>
       <c r="G8" s="30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H8" s="3"/>
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="28" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C9" s="28" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D9" s="29" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -3399,51 +3444,50 @@
   <dimension ref="A8:G9"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="21.85546875" style="49" customWidth="1"/>
-    <col min="2" max="2" width="66.28515625" style="49" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" style="49" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.85546875" style="49" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.140625" style="49" customWidth="1"/>
-    <col min="6" max="7" width="10.28515625" style="49" bestFit="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.140625" style="49"/>
+    <col min="1" max="1" width="21.85546875" customWidth="1"/>
+    <col min="2" max="2" width="66.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.140625" customWidth="1"/>
+    <col min="6" max="7" width="10.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="1:7">
-      <c r="A8" s="49" t="s">
+      <c r="A8" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="49" t="s">
+      <c r="B8" t="s">
         <v>49</v>
       </c>
-      <c r="C8" s="49" t="s">
+      <c r="C8" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="49" t="s">
+      <c r="D8" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="49" t="s">
+      <c r="E8" t="s">
         <v>53</v>
       </c>
-      <c r="F8" s="49" t="s">
-        <v>124</v>
+      <c r="F8" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="87">
-      <c r="A9" s="50" t="s">
-        <v>125</v>
-      </c>
-      <c r="B9" s="50" t="s">
+      <c r="A9" s="45" t="s">
         <v>126</v>
       </c>
-      <c r="C9" s="51" t="s">
-        <v>59</v>
-      </c>
-      <c r="D9" s="52"/>
-      <c r="E9" s="53" t="s">
+      <c r="B9" s="45" t="s">
         <v>127</v>
       </c>
-      <c r="F9" s="54"/>
-      <c r="G9" s="55"/>
+      <c r="C9" s="46" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="47" t="s">
+        <v>128</v>
+      </c>
+      <c r="F9" s="48"/>
+      <c r="G9" s="49"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -3475,22 +3519,22 @@
   <sheetData>
     <row r="2" spans="2:8">
       <c r="B2" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F2" s="10"/>
     </row>
     <row r="3" spans="2:8">
       <c r="B3" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E3" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -3498,149 +3542,149 @@
     </row>
     <row r="4" spans="2:8" ht="43.5">
       <c r="B4" s="2" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="5" spans="2:8" ht="102.75" customHeight="1">
       <c r="B5" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="6" spans="2:8" ht="43.5">
       <c r="B6" s="2" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="105.75" customHeight="1">
       <c r="B7" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="2:8" ht="64.5" customHeight="1">
       <c r="B8" s="2" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="2:8">
       <c r="B9" s="2" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="2:8">
       <c r="B10" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="2:8">
       <c r="B11" s="22" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C11" s="23" t="s">
         <v>40</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="12" spans="2:8">
       <c r="B12" s="25" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C12" s="23" t="s">
         <v>40</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E12" s="21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="13" spans="2:8">
       <c r="B13" s="22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C13" s="23" t="s">
         <v>40</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="2:8">
       <c r="B14" s="25" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C14" s="23" t="s">
         <v>40</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E14" s="21" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="2:8" ht="15">
       <c r="B15" s="2" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="18" spans="2:4">
@@ -3684,109 +3728,109 @@
   <sheetData>
     <row r="2" spans="2:5">
       <c r="B2" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D2" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" spans="2:5">
       <c r="B3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="2:5">
       <c r="B4" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="43.5">
       <c r="B5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C5" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="D5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="6" spans="2:5">
       <c r="B6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="2:5">
       <c r="B7" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C7" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D7" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="43.5">
       <c r="B8" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C8" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="9" spans="2:5">
       <c r="B9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="10" spans="2:5">
       <c r="B10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C10" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="12" spans="2:5">
       <c r="B12" s="27" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -3798,26 +3842,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -4024,8 +4048,28 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="bb18a1b9-ddba-4244-9634-64732d0cb267">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="06294a2e-6f87-4144-83b8-94a4d04d144a" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4033,5 +4077,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9D91DC9B-0D61-455B-BDC2-0A4F28AD2AEE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1ECF7AFC-EAC6-47C9-8578-0515052E4E5F}"/>
 </file>
</xml_diff>